<commit_message>
Add catalog History sheet and product timestamps
Backfill all 39 products as added on 2026-09-26 with stable
product ids plus created_at/modified_at in JSON and Excel.
</commit_message>
<xml_diff>
--- a/catalog/angaala-hub-product-catalog.xlsx
+++ b/catalog/angaala-hub-product-catalog.xlsx
@@ -8,8 +8,9 @@
   </bookViews>
   <sheets>
     <sheet name="Product Catalog" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Summary" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Unidentified Notes" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="History" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Summary" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Unidentified Notes" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Product Catalog'!$A$1:$G$40</definedName>
@@ -458,1495 +459,2098 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G40"/>
+  <dimension ref="A1:J40"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="22" customWidth="1" min="1" max="1"/>
-    <col width="48" customWidth="1" min="2" max="2"/>
-    <col width="14" customWidth="1" min="3" max="3"/>
-    <col width="55" customWidth="1" min="4" max="4"/>
-    <col width="55" customWidth="1" min="5" max="5"/>
-    <col width="55" customWidth="1" min="6" max="6"/>
-    <col width="55" customWidth="1" min="7" max="7"/>
+    <col width="18" customWidth="1" min="1" max="1"/>
+    <col width="18" customWidth="1" min="2" max="2"/>
+    <col width="18" customWidth="1" min="3" max="3"/>
+    <col width="18" customWidth="1" min="4" max="4"/>
+    <col width="18" customWidth="1" min="5" max="5"/>
+    <col width="18" customWidth="1" min="6" max="6"/>
+    <col width="40" customWidth="1" min="7" max="7"/>
+    <col width="18" customWidth="1" min="8" max="8"/>
+    <col width="18" customWidth="1" min="9" max="9"/>
+    <col width="18" customWidth="1" min="10" max="10"/>
   </cols>
   <sheetData>
     <row r="1" ht="22" customHeight="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" s="5" t="inlineStr">
+        <is>
+          <t>id</t>
+        </is>
+      </c>
+      <c r="B1" s="5" t="inlineStr">
         <is>
           <t>Category</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="C1" s="5" t="inlineStr">
         <is>
           <t>Product Name</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="D1" s="5" t="inlineStr">
         <is>
           <t>Price (INR)</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="E1" s="5" t="inlineStr">
         <is>
           <t>Image Source/URL</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="F1" s="5" t="inlineStr">
         <is>
           <t>Specs</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="G1" s="5" t="inlineStr">
         <is>
           <t>Notes</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="H1" s="5" t="inlineStr">
         <is>
           <t>Source Links</t>
         </is>
       </c>
+      <c r="I1" s="5" t="inlineStr">
+        <is>
+          <t>created_at</t>
+        </is>
+      </c>
+      <c r="J1" s="5" t="inlineStr">
+        <is>
+          <t>modified_at</t>
+        </is>
+      </c>
     </row>
     <row r="2">
-      <c r="A2" s="2" t="inlineStr">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>AH-001-infinix-smart-8-hd-shiny-gold-3gb-64gb</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
         <is>
           <t>Smartphones</t>
         </is>
       </c>
-      <c r="B2" s="2" t="inlineStr">
+      <c r="C2" t="inlineStr">
         <is>
           <t>Infinix SMART 8 HD (Shiny Gold, 3GB/64GB)</t>
         </is>
       </c>
-      <c r="C2" s="2" t="inlineStr">
+      <c r="D2" t="inlineStr">
         <is>
           <t>6699</t>
         </is>
       </c>
-      <c r="D2" s="2" t="inlineStr">
+      <c r="E2" t="inlineStr">
         <is>
           <t>/workspace/shakti-mobiles/images/products/phone-4g.jpg</t>
         </is>
       </c>
-      <c r="E2" s="2" t="inlineStr">
+      <c r="F2" t="inlineStr">
         <is>
           <t>6.6" HD+ IPS; Unisoc T606; 3GB RAM / 64GB ROM (expandable to 2TB); 13MP + AI rear, 8MP front; 5000mAh; 10W; Dual SIM 4G</t>
         </is>
       </c>
-      <c r="F2" s="2" t="inlineStr">
+      <c r="G2" t="inlineStr">
         <is>
           <t>Verified Flipkart listing. Color Shiny Gold visible in store product photo. Alternate images: phone-4g-infinix.jpg, phone-4g-alt.jpg.</t>
         </is>
       </c>
-      <c r="G2" s="2" t="inlineStr">
+      <c r="H2" t="inlineStr">
         <is>
           <t>https://www.flipkart.com/infinix-smart-8-hd-shiny-gold-64-gb/p/itm709d885ba6ac1?pid=MOBGVAPXG4WHFR9M ; https://infinixmobiles.in/products/smart-8-hd</t>
         </is>
       </c>
+      <c r="I2" t="inlineStr">
+        <is>
+          <t>2026-09-26T23:41:58+05:30</t>
+        </is>
+      </c>
+      <c r="J2" t="inlineStr">
+        <is>
+          <t>2026-09-26T23:41:58+05:30</t>
+        </is>
+      </c>
     </row>
     <row r="3">
-      <c r="A3" s="2" t="inlineStr">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>AH-002-poco-c75-5g-aqua-bliss-4gb-64gb</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
         <is>
           <t>Smartphones</t>
         </is>
       </c>
-      <c r="B3" s="2" t="inlineStr">
+      <c r="C3" t="inlineStr">
         <is>
           <t>POCO C75 5G (Aqua Bliss, 4GB/64GB)</t>
         </is>
       </c>
-      <c r="C3" s="2" t="inlineStr">
+      <c r="D3" t="inlineStr">
         <is>
           <t>10999</t>
         </is>
       </c>
-      <c r="D3" s="2" t="inlineStr">
+      <c r="E3" t="inlineStr">
         <is>
           <t>/workspace/shakti-mobiles/images/products/phone-5g-try1.jpg</t>
         </is>
       </c>
-      <c r="E3" s="2" t="inlineStr">
+      <c r="F3" t="inlineStr">
         <is>
           <t>6.88" HD+ 120Hz; Snapdragon 4s Gen 2 5G; 4GB/64GB (expandable 1TB); 50MP Sony rear, 5MP front; 5160mAh; Dual SIM</t>
         </is>
       </c>
-      <c r="F3" s="2" t="inlineStr">
+      <c r="G3" t="inlineStr">
         <is>
           <t>Prefer phone-5g-try1.jpg over phone-5g.jpg per catalog guidance. Flipkart ~INR 10,999 (bank offer may lower).</t>
         </is>
       </c>
-      <c r="G3" s="2" t="inlineStr">
+      <c r="H3" t="inlineStr">
         <is>
           <t>https://www.flipkart.com/poco-c75-5g-aqua-bliss-64-gb/p/itm10b3f6f1bc616</t>
         </is>
       </c>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>2026-09-26T23:41:58+05:30</t>
+        </is>
+      </c>
+      <c r="J3" t="inlineStr">
+        <is>
+          <t>2026-09-26T23:41:58+05:30</t>
+        </is>
+      </c>
     </row>
     <row r="4">
-      <c r="A4" s="2" t="inlineStr">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>AH-003-lava-bold-n4-lite-empire-gold-3gb-32gb</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
         <is>
           <t>Smartphones</t>
         </is>
       </c>
-      <c r="B4" s="2" t="inlineStr">
+      <c r="C4" t="inlineStr">
         <is>
           <t>Lava Bold N4 Lite (Empire Gold, 3GB/32GB)</t>
         </is>
       </c>
-      <c r="C4" s="2" t="inlineStr">
+      <c r="D4" t="inlineStr">
         <is>
           <t>8399</t>
         </is>
       </c>
-      <c r="D4" s="2" t="inlineStr">
+      <c r="E4" t="inlineStr">
         <is>
           <t>/workspace/shakti-mobiles/images/products/phone-samsung-f05.jpg</t>
         </is>
       </c>
-      <c r="E4" s="2" t="inlineStr">
+      <c r="F4" t="inlineStr">
         <is>
           <t>6.56" qHD; Unisoc 9863A; 3GB+3GB virtual RAM / 32GB ROM (expandable 64GB); 8MP rear, 5MP front; 5000mAh; 10W; Android 16 Go; MIL-STD-810H</t>
         </is>
       </c>
-      <c r="F4" s="2" t="inlineStr">
+      <c r="G4" t="inlineStr">
         <is>
           <t>File named phone-samsung-f05.jpg but image content is Lava Bold N4 Lite (LAVA logo + BOLD N4 LITE on screen). Same asset as phone-4g-samsung-amz.jpg. Amazon.in exclusive; ~INR 7,999–8,399.</t>
         </is>
       </c>
-      <c r="G4" s="2" t="inlineStr">
+      <c r="H4" t="inlineStr">
         <is>
           <t>https://www.amazon.in/Lava-Storage-Display-Fingerprint-Phone-Cover/dp/B0HDPDGKJ4 ; https://www.91mobiles.com/lava-bold-n4-lite-4g-price-in-india</t>
         </is>
       </c>
+      <c r="I4" t="inlineStr">
+        <is>
+          <t>2026-09-26T23:41:58+05:30</t>
+        </is>
+      </c>
+      <c r="J4" t="inlineStr">
+        <is>
+          <t>2026-09-26T23:41:58+05:30</t>
+        </is>
+      </c>
     </row>
     <row r="5">
-      <c r="A5" s="2" t="inlineStr">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>AH-004-samsung-galaxy-f05-4gb-64gb</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
         <is>
           <t>Smartphones</t>
         </is>
       </c>
-      <c r="B5" s="2" t="inlineStr">
+      <c r="C5" t="inlineStr">
         <is>
           <t>Samsung Galaxy F05 (4GB/64GB)</t>
         </is>
       </c>
-      <c r="C5" s="2" t="inlineStr">
+      <c r="D5" t="inlineStr">
         <is>
           <t>6499</t>
         </is>
       </c>
-      <c r="D5" s="2" t="inlineStr">
+      <c r="E5" t="inlineStr">
         <is>
           <t>Store brand signage (Samsung listed); no dedicated clear F05 product photo in inspected set</t>
         </is>
       </c>
-      <c r="E5" s="2" t="inlineStr">
+      <c r="F5" t="inlineStr">
         <is>
           <t>6.74" HD+; Helio G85; 4GB/64GB (expandable 1TB); 50MP+2MP rear, 8MP front; 5000mAh; 25W; Android 14; Dual SIM 4G</t>
         </is>
       </c>
-      <c r="F5" s="2" t="inlineStr">
+      <c r="G5" t="inlineStr">
         <is>
           <t>Store sells Samsung (signage). Prior catalog guidance confirmed ~INR 6,499 Flipkart/Smartprix. Dedicated image file was mislabeled (see Lava Bold N4 Lite row).</t>
         </is>
       </c>
-      <c r="G5" s="2" t="inlineStr">
+      <c r="H5" t="inlineStr">
         <is>
           <t>https://www.flipkart.com/samsung-galaxy-f05-twilight-blue-64-gb/p/itm84a914081ab93 ; https://www.smartprix.com/mobiles/samsung-galaxy-f05-ppd1u4z3r099</t>
         </is>
       </c>
+      <c r="I5" t="inlineStr">
+        <is>
+          <t>2026-09-26T23:41:58+05:30</t>
+        </is>
+      </c>
+      <c r="J5" t="inlineStr">
+        <is>
+          <t>2026-09-26T23:41:58+05:30</t>
+        </is>
+      </c>
     </row>
     <row r="6">
-      <c r="A6" s="2" t="inlineStr">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>AH-005-redmi-a3-assorted-variants</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
         <is>
           <t>Smartphones</t>
         </is>
       </c>
-      <c r="B6" s="2" t="inlineStr">
+      <c r="C6" t="inlineStr">
         <is>
           <t>REDMI A3 (assorted variants)</t>
         </is>
       </c>
-      <c r="C6" s="2" t="inlineStr">
+      <c r="D6" t="inlineStr">
         <is>
           <t>6998-7340</t>
         </is>
       </c>
-      <c r="D6" s="2" t="inlineStr">
+      <c r="E6" t="inlineStr">
         <is>
           <t>/workspace/shakti-mobiles/images/service-counter.jpg ; chat upload interior counter</t>
         </is>
       </c>
-      <c r="E6" s="2" t="inlineStr">
+      <c r="F6" t="inlineStr">
         <is>
           <t>Budget Redmi A-series; typical configs 3GB/64GB to 6GB/128GB; Dual SIM 4G</t>
         </is>
       </c>
-      <c r="F6" s="2" t="inlineStr">
+      <c r="G6" t="inlineStr">
         <is>
           <t>Red retail box clearly visible on glass counter labeled REDMI A3. Exact RAM/storage of in-store unit not readable; price range from Flipkart variants.</t>
         </is>
       </c>
-      <c r="G6" s="2" t="inlineStr">
+      <c r="H6" t="inlineStr">
         <is>
           <t>https://pricehistory.app/p/redmi-a3-lake-blue-64-gb-3-TTlxopmb ; https://www.flipkart.com/redmi-a3-lake-blue-128-gb/p/itmbe3bd4f2bebed</t>
         </is>
       </c>
+      <c r="I6" t="inlineStr">
+        <is>
+          <t>2026-09-26T23:41:58+05:30</t>
+        </is>
+      </c>
+      <c r="J6" t="inlineStr">
+        <is>
+          <t>2026-09-26T23:41:58+05:30</t>
+        </is>
+      </c>
     </row>
     <row r="7">
-      <c r="A7" s="2" t="inlineStr">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>AH-006-realme-smartphone-boxed-model-unclear</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
         <is>
           <t>Smartphones</t>
         </is>
       </c>
-      <c r="B7" s="2" t="inlineStr">
+      <c r="C7" t="inlineStr">
         <is>
           <t>realme smartphone (boxed — model unclear)</t>
         </is>
       </c>
-      <c r="C7" s="2" t="inlineStr">
+      <c r="D7" t="inlineStr">
         <is>
           <t>Varies</t>
         </is>
       </c>
-      <c r="D7" s="2" t="inlineStr">
+      <c r="E7" t="inlineStr">
         <is>
           <t>/workspace/shakti-mobiles/images/service-counter.jpg</t>
         </is>
       </c>
-      <c r="E7" s="2" t="inlineStr">
+      <c r="F7" t="inlineStr">
         <is>
           <t>realme branded yellow retail box on counter; exact model text not fully legible (possible C-series)</t>
         </is>
       </c>
-      <c r="F7" s="2" t="inlineStr">
+      <c r="G7" t="inlineStr">
         <is>
           <t>Could not confidently identify exact model from box photo. Store carries realme (signage + accessories).</t>
         </is>
       </c>
-      <c r="G7" s="2" t="inlineStr">
+      <c r="H7" t="inlineStr">
         <is>
           <t>https://www.realme.com/in/</t>
         </is>
       </c>
+      <c r="I7" t="inlineStr">
+        <is>
+          <t>2026-09-26T23:41:58+05:30</t>
+        </is>
+      </c>
+      <c r="J7" t="inlineStr">
+        <is>
+          <t>2026-09-26T23:41:58+05:30</t>
+        </is>
+      </c>
     </row>
     <row r="8">
-      <c r="A8" s="2" t="inlineStr">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>AH-007-nokia-feature-phone-105-110-class</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
         <is>
           <t>Feature Phones</t>
         </is>
       </c>
-      <c r="B8" s="2" t="inlineStr">
+      <c r="C8" t="inlineStr">
         <is>
           <t>Nokia feature phone (105/110-class)</t>
         </is>
       </c>
-      <c r="C8" s="2" t="inlineStr">
+      <c r="D8" t="inlineStr">
         <is>
           <t>999-1589</t>
         </is>
       </c>
-      <c r="D8" s="2" t="inlineStr">
+      <c r="E8" t="inlineStr">
         <is>
           <t>Chat upload service/accessory shelves (Nokia blue box)</t>
         </is>
       </c>
-      <c r="E8" s="2" t="inlineStr">
+      <c r="F8" t="inlineStr">
         <is>
           <t>Keypad feature phone; Dual SIM options typical for Nokia 105 Classic / related</t>
         </is>
       </c>
-      <c r="F8" s="2" t="inlineStr">
+      <c r="G8" t="inlineStr">
         <is>
           <t>Small blue Nokia retail box visible on lower accessory shelf. Exact SKU (105 vs 110) not readable at distance.</t>
         </is>
       </c>
-      <c r="G8" s="2" t="inlineStr">
+      <c r="H8" t="inlineStr">
         <is>
           <t>https://pricehunt.com/mobiles/nokia-105.php</t>
         </is>
       </c>
+      <c r="I8" t="inlineStr">
+        <is>
+          <t>2026-09-26T23:41:58+05:30</t>
+        </is>
+      </c>
+      <c r="J8" t="inlineStr">
+        <is>
+          <t>2026-09-26T23:41:58+05:30</t>
+        </is>
+      </c>
     </row>
     <row r="9">
-      <c r="A9" s="2" t="inlineStr">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>AH-008-assorted-fashion-back-covers-cartoon-glitter-but</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
         <is>
           <t>Phone Cases</t>
         </is>
       </c>
-      <c r="B9" s="2" t="inlineStr">
+      <c r="C9" t="inlineStr">
         <is>
           <t>Assorted fashion back covers (cartoon / glitter / butterfly)</t>
         </is>
       </c>
-      <c r="C9" s="2" t="inlineStr">
+      <c r="D9" t="inlineStr">
         <is>
           <t>99-499</t>
         </is>
       </c>
-      <c r="D9" s="2" t="inlineStr">
+      <c r="E9" t="inlineStr">
         <is>
           <t>/workspace/shakti-mobiles/images/cases-fashion.jpg ; chat fashion-case wall</t>
         </is>
       </c>
-      <c r="E9" s="2" t="inlineStr">
+      <c r="F9" t="inlineStr">
         <is>
           <t>TPU/silicone fashion cases; themes include Hello Kitty, Tom &amp; Jerry, Labubu, butterflies, glitter/quicksand, rhinestones</t>
         </is>
       </c>
-      <c r="F9" s="2" t="inlineStr">
+      <c r="G9" t="inlineStr">
         <is>
           <t>In-store assortment; price varies by model and style. Packaged as Fashion Case.</t>
         </is>
       </c>
-      <c r="G9" s="2" t="inlineStr">
+      <c r="H9" t="inlineStr">
         <is>
           <t>Typical India retail for generic fashion covers INR 99-499</t>
         </is>
       </c>
+      <c r="I9" t="inlineStr">
+        <is>
+          <t>2026-09-26T23:41:58+05:30</t>
+        </is>
+      </c>
+      <c r="J9" t="inlineStr">
+        <is>
+          <t>2026-09-26T23:41:58+05:30</t>
+        </is>
+      </c>
     </row>
     <row r="10">
-      <c r="A10" s="2" t="inlineStr">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>AH-009-geometric-diamond-facet-fashion-cases</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
         <is>
           <t>Phone Cases</t>
         </is>
       </c>
-      <c r="B10" s="2" t="inlineStr">
+      <c r="C10" t="inlineStr">
         <is>
           <t>Geometric / diamond-facet fashion cases</t>
         </is>
       </c>
-      <c r="C10" s="2" t="inlineStr">
+      <c r="D10" t="inlineStr">
         <is>
           <t>149-499</t>
         </is>
       </c>
-      <c r="D10" s="2" t="inlineStr">
+      <c r="E10" t="inlineStr">
         <is>
           <t>/workspace/shakti-mobiles/images/cases-fashion.jpg ; /workspace/shakti-mobiles/images/cases-wall.jpg</t>
         </is>
       </c>
-      <c r="E10" s="2" t="inlineStr">
+      <c r="F10" t="inlineStr">
         <is>
           <t>3D crystalline / mosaic facet hard-back fashion covers in pink, purple, gold, black</t>
         </is>
       </c>
-      <c r="F10" s="2" t="inlineStr">
+      <c r="G10" t="inlineStr">
         <is>
           <t>In-store assortment; price varies.</t>
         </is>
       </c>
-      <c r="G10" s="2" t="inlineStr">
+      <c r="H10" t="inlineStr">
         <is>
           <t>Typical India retail INR 149-499</t>
         </is>
       </c>
+      <c r="I10" t="inlineStr">
+        <is>
+          <t>2026-09-26T23:41:58+05:30</t>
+        </is>
+      </c>
+      <c r="J10" t="inlineStr">
+        <is>
+          <t>2026-09-26T23:41:58+05:30</t>
+        </is>
+      </c>
     </row>
     <row r="11">
-      <c r="A11" s="2" t="inlineStr">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>AH-010-transparent-tpu-clear-covers</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
         <is>
           <t>Phone Cases</t>
         </is>
       </c>
-      <c r="B11" s="2" t="inlineStr">
+      <c r="C11" t="inlineStr">
         <is>
           <t>Transparent TPU / clear covers</t>
         </is>
       </c>
-      <c r="C11" s="2" t="inlineStr">
+      <c r="D11" t="inlineStr">
         <is>
           <t>99-299</t>
         </is>
       </c>
-      <c r="D11" s="2" t="inlineStr">
+      <c r="E11" t="inlineStr">
         <is>
           <t>/workspace/shakti-mobiles/images/cases-wall.jpg ; interior counter glass case</t>
         </is>
       </c>
-      <c r="E11" s="2" t="inlineStr">
+      <c r="F11" t="inlineStr">
         <is>
           <t>Clear TPU/PC protective backs; some with glitter insert</t>
         </is>
       </c>
-      <c r="F11" s="2" t="inlineStr">
+      <c r="G11" t="inlineStr">
         <is>
           <t>Large wall inventory of basic clear covers. In-store assortment; price varies.</t>
         </is>
       </c>
-      <c r="G11" s="2" t="inlineStr">
+      <c r="H11" t="inlineStr">
         <is>
           <t>Typical India retail INR 99-299</t>
         </is>
       </c>
+      <c r="I11" t="inlineStr">
+        <is>
+          <t>2026-09-26T23:41:58+05:30</t>
+        </is>
+      </c>
+      <c r="J11" t="inlineStr">
+        <is>
+          <t>2026-09-26T23:41:58+05:30</t>
+        </is>
+      </c>
     </row>
     <row r="12">
-      <c r="A12" s="2" t="inlineStr">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>AH-011-lustre-rugged-matte-tpu-cases</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
         <is>
           <t>Phone Cases</t>
         </is>
       </c>
-      <c r="B12" s="2" t="inlineStr">
+      <c r="C12" t="inlineStr">
         <is>
           <t>Lustre rugged / matte TPU cases</t>
         </is>
       </c>
-      <c r="C12" s="2" t="inlineStr">
+      <c r="D12" t="inlineStr">
         <is>
           <t>199-499</t>
         </is>
       </c>
-      <c r="D12" s="2" t="inlineStr">
+      <c r="E12" t="inlineStr">
         <is>
           <t>/workspace/shakti-mobiles/images/cases-wall.jpg</t>
         </is>
       </c>
-      <c r="E12" s="2" t="inlineStr">
+      <c r="F12" t="inlineStr">
         <is>
           <t>Lustre-branded yellow/black hang packs; solid black/navy/red matte or textured protective covers</t>
         </is>
       </c>
-      <c r="F12" s="2" t="inlineStr">
+      <c r="G12" t="inlineStr">
         <is>
           <t>Brand Lustre visible on packaging. Premium end of in-store case range.</t>
         </is>
       </c>
-      <c r="G12" s="2" t="inlineStr">
+      <c r="H12" t="inlineStr">
         <is>
           <t>Typical India retail for branded rugged TPU INR 199-499</t>
         </is>
       </c>
+      <c r="I12" t="inlineStr">
+        <is>
+          <t>2026-09-26T23:41:58+05:30</t>
+        </is>
+      </c>
+      <c r="J12" t="inlineStr">
+        <is>
+          <t>2026-09-26T23:41:58+05:30</t>
+        </is>
+      </c>
     </row>
     <row r="13">
-      <c r="A13" s="2" t="inlineStr">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>AH-012-magsafe-compatible-clear-cases</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
         <is>
           <t>Phone Cases</t>
         </is>
       </c>
-      <c r="B13" s="2" t="inlineStr">
+      <c r="C13" t="inlineStr">
         <is>
           <t>MagSafe-compatible clear cases</t>
         </is>
       </c>
-      <c r="C13" s="2" t="inlineStr">
+      <c r="D13" t="inlineStr">
         <is>
           <t>299-499</t>
         </is>
       </c>
-      <c r="D13" s="2" t="inlineStr">
+      <c r="E13" t="inlineStr">
         <is>
           <t>/workspace/shakti-mobiles/images/cases-wall.jpg</t>
         </is>
       </c>
-      <c r="E13" s="2" t="inlineStr">
+      <c r="F13" t="inlineStr">
         <is>
           <t>Clear cases with white circular MagSafe-style magnetic ring</t>
         </is>
       </c>
-      <c r="F13" s="2" t="inlineStr">
+      <c r="G13" t="inlineStr">
         <is>
           <t>Multiple MagSafe ring cases on wall pegs. In-store assortment.</t>
         </is>
       </c>
-      <c r="G13" s="2" t="inlineStr">
+      <c r="H13" t="inlineStr">
         <is>
           <t>Typical India retail INR 299-499</t>
         </is>
       </c>
+      <c r="I13" t="inlineStr">
+        <is>
+          <t>2026-09-26T23:41:58+05:30</t>
+        </is>
+      </c>
+      <c r="J13" t="inlineStr">
+        <is>
+          <t>2026-09-26T23:41:58+05:30</t>
+        </is>
+      </c>
     </row>
     <row r="14">
-      <c r="A14" s="2" t="inlineStr">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>AH-013-puffer-quilted-jacket-style-cases</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
         <is>
           <t>Phone Cases</t>
         </is>
       </c>
-      <c r="B14" s="2" t="inlineStr">
+      <c r="C14" t="inlineStr">
         <is>
           <t>Puffer / quilted jacket-style cases</t>
         </is>
       </c>
-      <c r="C14" s="2" t="inlineStr">
+      <c r="D14" t="inlineStr">
         <is>
           <t>249-499</t>
         </is>
       </c>
-      <c r="D14" s="2" t="inlineStr">
+      <c r="E14" t="inlineStr">
         <is>
           <t>/workspace/shakti-mobiles/images/cases-wall.jpg</t>
         </is>
       </c>
-      <c r="E14" s="2" t="inlineStr">
+      <c r="F14" t="inlineStr">
         <is>
           <t>Quilted puffer textured soft cases, typically black</t>
         </is>
       </c>
-      <c r="F14" s="2" t="inlineStr">
+      <c r="G14" t="inlineStr">
         <is>
           <t>At least two puffer-style units visible on cases wall.</t>
         </is>
       </c>
-      <c r="G14" s="2" t="inlineStr">
+      <c r="H14" t="inlineStr">
         <is>
           <t>Typical India retail INR 249-499</t>
         </is>
       </c>
+      <c r="I14" t="inlineStr">
+        <is>
+          <t>2026-09-26T23:41:58+05:30</t>
+        </is>
+      </c>
+      <c r="J14" t="inlineStr">
+        <is>
+          <t>2026-09-26T23:41:58+05:30</t>
+        </is>
+      </c>
     </row>
     <row r="15">
-      <c r="A15" s="2" t="inlineStr">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>AH-014-designer-character-graphic-cases-disney-luxury-m</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
         <is>
           <t>Phone Cases</t>
         </is>
       </c>
-      <c r="B15" s="2" t="inlineStr">
+      <c r="C15" t="inlineStr">
         <is>
           <t>Designer / character graphic cases (Disney, luxury-motif prints)</t>
         </is>
       </c>
-      <c r="C15" s="2" t="inlineStr">
+      <c r="D15" t="inlineStr">
         <is>
           <t>149-499</t>
         </is>
       </c>
-      <c r="D15" s="2" t="inlineStr">
+      <c r="E15" t="inlineStr">
         <is>
           <t>/workspace/shakti-mobiles/images/cases-wall.jpg</t>
         </is>
       </c>
-      <c r="E15" s="2" t="inlineStr">
+      <c r="F15" t="inlineStr">
         <is>
           <t>Printed graphic covers including Disney (Donald Duck, Minnie), Chanel/Dior-style motifs, Starbucks-style, Ferrari-style logos</t>
         </is>
       </c>
-      <c r="F15" s="2" t="inlineStr">
+      <c r="G15" t="inlineStr">
         <is>
           <t>In-store assortment of printed designer-look cases; unofficial motif prints common in local retail.</t>
         </is>
       </c>
-      <c r="G15" s="2" t="inlineStr">
+      <c r="H15" t="inlineStr">
         <is>
           <t>Typical India retail INR 149-499</t>
         </is>
       </c>
+      <c r="I15" t="inlineStr">
+        <is>
+          <t>2026-09-26T23:41:58+05:30</t>
+        </is>
+      </c>
+      <c r="J15" t="inlineStr">
+        <is>
+          <t>2026-09-26T23:41:58+05:30</t>
+        </is>
+      </c>
     </row>
     <row r="16">
-      <c r="A16" s="2" t="inlineStr">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>AH-015-yellow-waterproof-phone-pouches-dry-bags-with-la</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
         <is>
           <t>Phone Accessories</t>
         </is>
       </c>
-      <c r="B16" s="2" t="inlineStr">
+      <c r="C16" t="inlineStr">
         <is>
           <t>Yellow waterproof phone pouches (dry bags with lanyard)</t>
         </is>
       </c>
-      <c r="C16" s="2" t="inlineStr">
+      <c r="D16" t="inlineStr">
         <is>
           <t>99-249</t>
         </is>
       </c>
-      <c r="D16" s="2" t="inlineStr">
+      <c r="E16" t="inlineStr">
         <is>
           <t>/workspace/shakti-mobiles/images/cases-wall.jpg</t>
         </is>
       </c>
-      <c r="E16" s="2" t="inlineStr">
+      <c r="F16" t="inlineStr">
         <is>
           <t>Transparent yellow waterproof dry bag with matching neck lanyard; universal phone size</t>
         </is>
       </c>
-      <c r="F16" s="2" t="inlineStr">
+      <c r="G16" t="inlineStr">
         <is>
           <t>Cluster hanging on far-right of cases wall. In-store assortment.</t>
         </is>
       </c>
-      <c r="G16" s="2" t="inlineStr">
+      <c r="H16" t="inlineStr">
         <is>
           <t>Typical India retail waterproof pouches INR 99-249</t>
         </is>
       </c>
+      <c r="I16" t="inlineStr">
+        <is>
+          <t>2026-09-26T23:41:58+05:30</t>
+        </is>
+      </c>
+      <c r="J16" t="inlineStr">
+        <is>
+          <t>2026-09-26T23:41:58+05:30</t>
+        </is>
+      </c>
     </row>
     <row r="17">
-      <c r="A17" s="2" t="inlineStr">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>AH-016-tempered-glass-screen-protector</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
         <is>
           <t>Screen Protection</t>
         </is>
       </c>
-      <c r="B17" s="2" t="inlineStr">
+      <c r="C17" t="inlineStr">
         <is>
           <t>Tempered glass screen protector</t>
         </is>
       </c>
-      <c r="C17" s="2" t="inlineStr">
+      <c r="D17" t="inlineStr">
         <is>
           <t>100</t>
         </is>
       </c>
-      <c r="D17" s="2" t="inlineStr">
+      <c r="E17" t="inlineStr">
         <is>
           <t>/workspace/shakti-mobiles/images/storefront-1.jpg ; storefront-2.jpg</t>
         </is>
       </c>
-      <c r="E17" s="2" t="inlineStr">
+      <c r="F17" t="inlineStr">
         <is>
           <t>Generic tempered glass; store advertises base price INR 100</t>
         </is>
       </c>
-      <c r="F17" s="2" t="inlineStr">
+      <c r="G17" t="inlineStr">
         <is>
           <t>Window card: ANGAALA HUB TEMPER GLASS INR 100. Model-specific pricing may vary.</t>
         </is>
       </c>
-      <c r="G17" s="2" t="inlineStr">
+      <c r="H17" t="inlineStr">
         <is>
           <t>In-store advertised price INR 100</t>
         </is>
       </c>
+      <c r="I17" t="inlineStr">
+        <is>
+          <t>2026-09-26T23:41:58+05:30</t>
+        </is>
+      </c>
+      <c r="J17" t="inlineStr">
+        <is>
+          <t>2026-09-26T23:41:58+05:30</t>
+        </is>
+      </c>
     </row>
     <row r="18">
-      <c r="A18" s="2" t="inlineStr">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>AH-017-custom-cut-screen-guard-uv-film-auto-laminate-ma</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
         <is>
           <t>Screen Protection</t>
         </is>
       </c>
-      <c r="B18" s="2" t="inlineStr">
+      <c r="C18" t="inlineStr">
         <is>
           <t>Custom-cut screen guard / UV film (auto laminate machine)</t>
         </is>
       </c>
-      <c r="C18" s="2" t="inlineStr">
+      <c r="D18" t="inlineStr">
         <is>
           <t>149-499</t>
         </is>
       </c>
-      <c r="D18" s="2" t="inlineStr">
+      <c r="E18" t="inlineStr">
         <is>
           <t>Chat upload counter (REPROTECT UV vacuum film applicator); storefront yellow banner</t>
         </is>
       </c>
-      <c r="E18" s="2" t="inlineStr">
+      <c r="F18" t="inlineStr">
         <is>
           <t>Sticker/screen guard cutting machine with auto laminate; UV curing lamp; matte/glossy options; mobile + laptop skins</t>
         </is>
       </c>
-      <c r="F18" s="2" t="inlineStr">
+      <c r="G18" t="inlineStr">
         <is>
           <t>REPROTECT Mobile UV vacuum film applicator under glass counter. Service + product hybrid.</t>
         </is>
       </c>
-      <c r="G18" s="2" t="inlineStr">
+      <c r="H18" t="inlineStr">
         <is>
           <t>Typical India custom hydrogel/UV film installs INR 149-499</t>
         </is>
       </c>
+      <c r="I18" t="inlineStr">
+        <is>
+          <t>2026-09-26T23:41:58+05:30</t>
+        </is>
+      </c>
+      <c r="J18" t="inlineStr">
+        <is>
+          <t>2026-09-26T23:41:58+05:30</t>
+        </is>
+      </c>
     </row>
     <row r="19">
-      <c r="A19" s="2" t="inlineStr">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>AH-018-laptop-and-mobile-skins</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
         <is>
           <t>Screen Protection</t>
         </is>
       </c>
-      <c r="B19" s="2" t="inlineStr">
+      <c r="C19" t="inlineStr">
         <is>
           <t>Laptop and mobile skins</t>
         </is>
       </c>
-      <c r="C19" s="2" t="inlineStr">
+      <c r="D19" t="inlineStr">
         <is>
           <t>149-499</t>
         </is>
       </c>
-      <c r="D19" s="2" t="inlineStr">
+      <c r="E19" t="inlineStr">
         <is>
           <t>/workspace/shakti-mobiles/images/storefront-1.jpg</t>
         </is>
       </c>
-      <c r="E19" s="2" t="inlineStr">
+      <c r="F19" t="inlineStr">
         <is>
           <t>Adhesive decorative/protective skins for phones and laptops</t>
         </is>
       </c>
-      <c r="F19" s="2" t="inlineStr">
+      <c r="G19" t="inlineStr">
         <is>
           <t>Blue flyer in window: Laptop and Mobile Skins.</t>
         </is>
       </c>
-      <c r="G19" s="2" t="inlineStr">
+      <c r="H19" t="inlineStr">
         <is>
           <t>Typical India retail skins INR 149-499</t>
         </is>
       </c>
+      <c r="I19" t="inlineStr">
+        <is>
+          <t>2026-09-26T23:41:58+05:30</t>
+        </is>
+      </c>
+      <c r="J19" t="inlineStr">
+        <is>
+          <t>2026-09-26T23:41:58+05:30</t>
+        </is>
+      </c>
     </row>
     <row r="20">
-      <c r="A20" s="2" t="inlineStr">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>AH-019-boat-rockerz-450-on-ear-bluetooth</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
         <is>
           <t>Audio - Headphones</t>
         </is>
       </c>
-      <c r="B20" s="2" t="inlineStr">
+      <c r="C20" t="inlineStr">
         <is>
           <t>boAt Rockerz 450 (on-ear Bluetooth)</t>
         </is>
       </c>
-      <c r="C20" s="2" t="inlineStr">
+      <c r="D20" t="inlineStr">
         <is>
           <t>1699-1899</t>
         </is>
       </c>
-      <c r="D20" s="2" t="inlineStr">
+      <c r="E20" t="inlineStr">
         <is>
           <t>/workspace/shakti-mobiles/images/interior-counter.jpg</t>
         </is>
       </c>
-      <c r="E20" s="2" t="inlineStr">
+      <c r="F20" t="inlineStr">
         <is>
           <t>40mm drivers; up to ~15H playback; Bluetooth + AUX; on-ear</t>
         </is>
       </c>
-      <c r="F20" s="2" t="inlineStr">
+      <c r="G20" t="inlineStr">
         <is>
           <t>White boAt over-ear/on-ear box visible on top accessory shelf.</t>
         </is>
       </c>
-      <c r="G20" s="2" t="inlineStr">
+      <c r="H20" t="inlineStr">
         <is>
           <t>https://www.boat-lifestyle.com/products/rockerz-450 ; https://www.flipkart.com/boat-rockerz-450-40mm-drivers-15h-battery-stream-ad-free-music-via-app-bluetooth/p/itm077a566bd128b</t>
         </is>
       </c>
+      <c r="I20" t="inlineStr">
+        <is>
+          <t>2026-09-26T23:41:58+05:30</t>
+        </is>
+      </c>
+      <c r="J20" t="inlineStr">
+        <is>
+          <t>2026-09-26T23:41:58+05:30</t>
+        </is>
+      </c>
     </row>
     <row r="21">
-      <c r="A21" s="2" t="inlineStr">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>AH-020-boat-shine-assorted-over-ear-headphones</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
         <is>
           <t>Audio - Headphones</t>
         </is>
       </c>
-      <c r="B21" s="2" t="inlineStr">
+      <c r="C21" t="inlineStr">
         <is>
           <t>boAt Shine / assorted over-ear headphones</t>
         </is>
       </c>
-      <c r="C21" s="2" t="inlineStr">
+      <c r="D21" t="inlineStr">
         <is>
           <t>1499-2499</t>
         </is>
       </c>
-      <c r="D21" s="2" t="inlineStr">
+      <c r="E21" t="inlineStr">
         <is>
           <t>Chat upload accessory shelves; interior-counter.jpg</t>
         </is>
       </c>
-      <c r="E21" s="2" t="inlineStr">
+      <c r="F21" t="inlineStr">
         <is>
           <t>Over-ear wireless headphones; boAt Shine white/silver packaging among others (P9/P3 wireless headsets also stocked)</t>
         </is>
       </c>
-      <c r="F21" s="2" t="inlineStr">
+      <c r="G21" t="inlineStr">
         <is>
           <t>Multiple over-ear boxes on top shelf including boAt Shine, P9 Wireless Headset, Noise headphones.</t>
         </is>
       </c>
-      <c r="G21" s="2" t="inlineStr">
+      <c r="H21" t="inlineStr">
         <is>
           <t>Typical India retail over-ear Bluetooth INR 1499-2499</t>
         </is>
       </c>
+      <c r="I21" t="inlineStr">
+        <is>
+          <t>2026-09-26T23:41:58+05:30</t>
+        </is>
+      </c>
+      <c r="J21" t="inlineStr">
+        <is>
+          <t>2026-09-26T23:41:58+05:30</t>
+        </is>
+      </c>
     </row>
     <row r="22">
-      <c r="A22" s="2" t="inlineStr">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>AH-021-boat-rockerz-series-wireless-neckbands-assorted</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
         <is>
           <t>Audio - Neckbands</t>
         </is>
       </c>
-      <c r="B22" s="2" t="inlineStr">
+      <c r="C22" t="inlineStr">
         <is>
           <t>boAt Rockerz series wireless neckbands (assorted)</t>
         </is>
       </c>
-      <c r="C22" s="2" t="inlineStr">
+      <c r="D22" t="inlineStr">
         <is>
           <t>799-1499</t>
         </is>
       </c>
-      <c r="D22" s="2" t="inlineStr">
+      <c r="E22" t="inlineStr">
         <is>
           <t>/workspace/shakti-mobiles/images/interior-counter.jpg ; service-counter.jpg</t>
         </is>
       </c>
-      <c r="E22" s="2" t="inlineStr">
+      <c r="F22" t="inlineStr">
         <is>
           <t>Wireless neckband earphones; Rockerz / Rockerz Turbo Power lineup; Bluetooth</t>
         </is>
       </c>
-      <c r="F22" s="2" t="inlineStr">
+      <c r="G22" t="inlineStr">
         <is>
           <t>Many slim boAt Rockerz boxes; Hardik Pandya Rockerz Turbo Power standee visible. Also Captain / Vibration branded neckband boxes.</t>
         </is>
       </c>
-      <c r="G22" s="2" t="inlineStr">
+      <c r="H22" t="inlineStr">
         <is>
           <t>https://www.boat-lifestyle.com/ ; Flipkart boAt Rockerz listings typically INR 799-1499</t>
         </is>
       </c>
+      <c r="I22" t="inlineStr">
+        <is>
+          <t>2026-09-26T23:41:58+05:30</t>
+        </is>
+      </c>
+      <c r="J22" t="inlineStr">
+        <is>
+          <t>2026-09-26T23:41:58+05:30</t>
+        </is>
+      </c>
     </row>
     <row r="23">
-      <c r="A23" s="2" t="inlineStr">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>AH-022-noise-wireless-neckband</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
         <is>
           <t>Audio - Neckbands</t>
         </is>
       </c>
-      <c r="B23" s="2" t="inlineStr">
+      <c r="C23" t="inlineStr">
         <is>
           <t>Noise wireless neckband</t>
         </is>
       </c>
-      <c r="C23" s="2" t="inlineStr">
+      <c r="D23" t="inlineStr">
         <is>
           <t>999-1499</t>
         </is>
       </c>
-      <c r="D23" s="2" t="inlineStr">
+      <c r="E23" t="inlineStr">
         <is>
           <t>Chat upload accessory shelves; interior-counter.jpg</t>
         </is>
       </c>
-      <c r="E23" s="2" t="inlineStr">
+      <c r="F23" t="inlineStr">
         <is>
           <t>Noise-branded wireless neckband earphones</t>
         </is>
       </c>
-      <c r="F23" s="2" t="inlineStr">
+      <c r="G23" t="inlineStr">
         <is>
           <t>Light blue / black Noise box on audio shelf. Exact model name not fully readable.</t>
         </is>
       </c>
-      <c r="G23" s="2" t="inlineStr">
+      <c r="H23" t="inlineStr">
         <is>
           <t>https://www.smartprix.com/mobile_headphones/noise-nerve-wireless-neckband-ppd146xzqfsb</t>
         </is>
       </c>
+      <c r="I23" t="inlineStr">
+        <is>
+          <t>2026-09-26T23:41:58+05:30</t>
+        </is>
+      </c>
+      <c r="J23" t="inlineStr">
+        <is>
+          <t>2026-09-26T23:41:58+05:30</t>
+        </is>
+      </c>
     </row>
     <row r="24">
-      <c r="A24" s="2" t="inlineStr">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>AH-023-ditto-rockers-13-pro-neckbands</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
         <is>
           <t>Audio - Neckbands</t>
         </is>
       </c>
-      <c r="B24" s="2" t="inlineStr">
+      <c r="C24" t="inlineStr">
         <is>
           <t>DITTO / Rockers 13 Pro neckbands</t>
         </is>
       </c>
-      <c r="C24" s="2" t="inlineStr">
+      <c r="D24" t="inlineStr">
         <is>
           <t>499-999</t>
         </is>
       </c>
-      <c r="D24" s="2" t="inlineStr">
+      <c r="E24" t="inlineStr">
         <is>
           <t>/workspace/shakti-mobiles/images/interior-counter.jpg</t>
         </is>
       </c>
-      <c r="E24" s="2" t="inlineStr">
+      <c r="F24" t="inlineStr">
         <is>
           <t>Value wireless neckbands; Rockers 13 Pro box advertises long playback (e.g. 450h claim on pack)</t>
         </is>
       </c>
-      <c r="F24" s="2" t="inlineStr">
+      <c r="G24" t="inlineStr">
         <is>
           <t>Local/value brands alongside boAt on same shelves.</t>
         </is>
       </c>
-      <c r="G24" s="2" t="inlineStr">
+      <c r="H24" t="inlineStr">
         <is>
           <t>Typical India retail value neckbands INR 499-999</t>
         </is>
       </c>
+      <c r="I24" t="inlineStr">
+        <is>
+          <t>2026-09-26T23:41:58+05:30</t>
+        </is>
+      </c>
+      <c r="J24" t="inlineStr">
+        <is>
+          <t>2026-09-26T23:41:58+05:30</t>
+        </is>
+      </c>
     </row>
     <row r="25">
-      <c r="A25" s="2" t="inlineStr">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>AH-024-realme-buds-wireless-buds-classic-neckband-and-w</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
         <is>
           <t>Audio - Neckbands</t>
         </is>
       </c>
-      <c r="B25" s="2" t="inlineStr">
+      <c r="C25" t="inlineStr">
         <is>
           <t>realme Buds Wireless / Buds Classic (neckband and wired)</t>
         </is>
       </c>
-      <c r="C25" s="2" t="inlineStr">
+      <c r="D25" t="inlineStr">
         <is>
           <t>699-1499</t>
         </is>
       </c>
-      <c r="D25" s="2" t="inlineStr">
+      <c r="E25" t="inlineStr">
         <is>
           <t>/workspace/shakti-mobiles/images/interior-counter.jpg</t>
         </is>
       </c>
-      <c r="E25" s="2" t="inlineStr">
+      <c r="F25" t="inlineStr">
         <is>
           <t>realme yellow retail audio boxes; Buds Classic wired and Buds Wireless neckband variants stocked</t>
         </is>
       </c>
-      <c r="F25" s="2" t="inlineStr">
+      <c r="G25" t="inlineStr">
         <is>
           <t>Multiple signature yellow realme audio boxes on charger/TWS shelf row.</t>
         </is>
       </c>
-      <c r="G25" s="2" t="inlineStr">
+      <c r="H25" t="inlineStr">
         <is>
           <t>Flipkart realme Buds listings typically INR 699-1499</t>
         </is>
       </c>
+      <c r="I25" t="inlineStr">
+        <is>
+          <t>2026-09-26T23:41:58+05:30</t>
+        </is>
+      </c>
+      <c r="J25" t="inlineStr">
+        <is>
+          <t>2026-09-26T23:41:58+05:30</t>
+        </is>
+      </c>
     </row>
     <row r="26">
-      <c r="A26" s="2" t="inlineStr">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>AH-025-oneplus-nord-buds-2r-buds-2r</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
         <is>
           <t>Audio - TWS Earbuds</t>
         </is>
       </c>
-      <c r="B26" s="2" t="inlineStr">
+      <c r="C26" t="inlineStr">
         <is>
           <t>OnePlus Nord Buds 2r (Buds 2r)</t>
         </is>
       </c>
-      <c r="C26" s="2" t="inlineStr">
+      <c r="D26" t="inlineStr">
         <is>
           <t>1649-2199</t>
         </is>
       </c>
-      <c r="D26" s="2" t="inlineStr">
+      <c r="E26" t="inlineStr">
         <is>
           <t>Chat upload accessory shelves; interior-counter.jpg</t>
         </is>
       </c>
-      <c r="E26" s="2" t="inlineStr">
+      <c r="F26" t="inlineStr">
         <is>
           <t>True wireless earbuds; OnePlus Buds 2r / Nord Buds 2R packaging</t>
         </is>
       </c>
-      <c r="F26" s="2" t="inlineStr">
+      <c r="G26" t="inlineStr">
         <is>
           <t>White/blue Buds 2r box visible among TWS row.</t>
         </is>
       </c>
-      <c r="G26" s="2" t="inlineStr">
+      <c r="H26" t="inlineStr">
         <is>
           <t>https://www.smartprix.com/mobile_headphones/oneplus-nord-buds-2r-true-wireless-earbuds-ppd15t83jbh5</t>
         </is>
       </c>
+      <c r="I26" t="inlineStr">
+        <is>
+          <t>2026-09-26T23:41:58+05:30</t>
+        </is>
+      </c>
+      <c r="J26" t="inlineStr">
+        <is>
+          <t>2026-09-26T23:41:58+05:30</t>
+        </is>
+      </c>
     </row>
     <row r="27">
-      <c r="A27" s="2" t="inlineStr">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>AH-026-boat-airdopes-tws-assorted-models</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
         <is>
           <t>Audio - TWS Earbuds</t>
         </is>
       </c>
-      <c r="B27" s="2" t="inlineStr">
+      <c r="C27" t="inlineStr">
         <is>
           <t>boAt Airdopes TWS (assorted models)</t>
         </is>
       </c>
-      <c r="C27" s="2" t="inlineStr">
+      <c r="D27" t="inlineStr">
         <is>
           <t>799-1999</t>
         </is>
       </c>
-      <c r="D27" s="2" t="inlineStr">
+      <c r="E27" t="inlineStr">
         <is>
           <t>/workspace/shakti-mobiles/images/interior-counter.jpg</t>
         </is>
       </c>
-      <c r="E27" s="2" t="inlineStr">
+      <c r="F27" t="inlineStr">
         <is>
           <t>boAt Airdopes true wireless earbuds; multiple SKUs on shelf</t>
         </is>
       </c>
-      <c r="F27" s="2" t="inlineStr">
+      <c r="G27" t="inlineStr">
         <is>
           <t>Several small Airdopes boxes on TWS shelf. Exact model mix varies.</t>
         </is>
       </c>
-      <c r="G27" s="2" t="inlineStr">
+      <c r="H27" t="inlineStr">
         <is>
           <t>https://www.boat-lifestyle.com/ ; Flipkart Airdopes typically INR 799-1999</t>
         </is>
       </c>
+      <c r="I27" t="inlineStr">
+        <is>
+          <t>2026-09-26T23:41:58+05:30</t>
+        </is>
+      </c>
+      <c r="J27" t="inlineStr">
+        <is>
+          <t>2026-09-26T23:41:58+05:30</t>
+        </is>
+      </c>
     </row>
     <row r="28">
-      <c r="A28" s="2" t="inlineStr">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>AH-027-u-i-m10-generic-tws-earbuds</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
         <is>
           <t>Audio - TWS Earbuds</t>
         </is>
       </c>
-      <c r="B28" s="2" t="inlineStr">
+      <c r="C28" t="inlineStr">
         <is>
           <t>U&amp;i / M10 / generic TWS earbuds</t>
         </is>
       </c>
-      <c r="C28" s="2" t="inlineStr">
+      <c r="D28" t="inlineStr">
         <is>
           <t>499-999</t>
         </is>
       </c>
-      <c r="D28" s="2" t="inlineStr">
+      <c r="E28" t="inlineStr">
         <is>
           <t>/workspace/shakti-mobiles/images/interior-counter.jpg</t>
         </is>
       </c>
-      <c r="E28" s="2" t="inlineStr">
+      <c r="F28" t="inlineStr">
         <is>
           <t>Value TWS earbuds (U&amp;i branded and M10-style packs)</t>
         </is>
       </c>
-      <c r="F28" s="2" t="inlineStr">
+      <c r="G28" t="inlineStr">
         <is>
           <t>Value TWS next to branded boAt/OnePlus stock.</t>
         </is>
       </c>
-      <c r="G28" s="2" t="inlineStr">
+      <c r="H28" t="inlineStr">
         <is>
           <t>Typical India retail generic TWS INR 499-999</t>
         </is>
       </c>
+      <c r="I28" t="inlineStr">
+        <is>
+          <t>2026-09-26T23:41:58+05:30</t>
+        </is>
+      </c>
+      <c r="J28" t="inlineStr">
+        <is>
+          <t>2026-09-26T23:41:58+05:30</t>
+        </is>
+      </c>
     </row>
     <row r="29">
-      <c r="A29" s="2" t="inlineStr">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>AH-028-lyne-jukebox-18-blaster-party-speaker</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
         <is>
           <t>Audio - Speakers</t>
         </is>
       </c>
-      <c r="B29" s="2" t="inlineStr">
+      <c r="C29" t="inlineStr">
         <is>
           <t>LYNE JukeBox 18 / Blaster party speaker</t>
         </is>
       </c>
-      <c r="C29" s="2" t="inlineStr">
+      <c r="D29" t="inlineStr">
         <is>
           <t>1899-1999</t>
         </is>
       </c>
-      <c r="D29" s="2" t="inlineStr">
+      <c r="E29" t="inlineStr">
         <is>
           <t>/workspace/shakti-mobiles/images/storefront-1.jpg ; storefront-2.jpg</t>
         </is>
       </c>
-      <c r="E29" s="2" t="inlineStr">
+      <c r="F29" t="inlineStr">
         <is>
           <t>~30-50W wireless party speaker; dual drivers; RGB lighting; Bluetooth; some kits include mic</t>
         </is>
       </c>
-      <c r="F29" s="2" t="inlineStr">
+      <c r="G29" t="inlineStr">
         <is>
           <t>Large LYNE JukeBox / Blaster boxes in front window. JukeBox 18 Pro launch around INR 1999.</t>
         </is>
       </c>
-      <c r="G29" s="2" t="inlineStr">
+      <c r="H29" t="inlineStr">
         <is>
           <t>https://lyneoriginals.com/products/jukebox-18 ; https://www.fonearena.com/blog/488457/lyne-blaster-series-jukebox-18-pro-price-features.html</t>
         </is>
       </c>
+      <c r="I29" t="inlineStr">
+        <is>
+          <t>2026-09-26T23:41:58+05:30</t>
+        </is>
+      </c>
+      <c r="J29" t="inlineStr">
+        <is>
+          <t>2026-09-26T23:41:58+05:30</t>
+        </is>
+      </c>
     </row>
     <row r="30">
-      <c r="A30" s="2" t="inlineStr">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>AH-029-lyne-blast-max-large-portable-bluetooth-speaker</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
         <is>
           <t>Audio - Speakers</t>
         </is>
       </c>
-      <c r="B30" s="2" t="inlineStr">
+      <c r="C30" t="inlineStr">
         <is>
           <t>LYNE BLAST MAX / large portable Bluetooth speaker</t>
         </is>
       </c>
-      <c r="C30" s="2" t="inlineStr">
+      <c r="D30" t="inlineStr">
         <is>
           <t>1499-2499</t>
         </is>
       </c>
-      <c r="D30" s="2" t="inlineStr">
+      <c r="E30" t="inlineStr">
         <is>
           <t>/workspace/shakti-mobiles/images/storefront-1.jpg</t>
         </is>
       </c>
-      <c r="E30" s="2" t="inlineStr">
+      <c r="F30" t="inlineStr">
         <is>
           <t>Large vertical portable Bluetooth speaker; dual-woofer party style with RGB rings (window display)</t>
         </is>
       </c>
-      <c r="F30" s="2" t="inlineStr">
+      <c r="G30" t="inlineStr">
         <is>
           <t>BLAST MAX and similar large speaker boxes in storefront window.</t>
         </is>
       </c>
-      <c r="G30" s="2" t="inlineStr">
+      <c r="H30" t="inlineStr">
         <is>
           <t>LYNE / local portable speaker retail typically INR 1499-2499</t>
         </is>
       </c>
+      <c r="I30" t="inlineStr">
+        <is>
+          <t>2026-09-26T23:41:58+05:30</t>
+        </is>
+      </c>
+      <c r="J30" t="inlineStr">
+        <is>
+          <t>2026-09-26T23:41:58+05:30</t>
+        </is>
+      </c>
     </row>
     <row r="31">
-      <c r="A31" s="2" t="inlineStr">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>AH-030-aeromic-mobile-wireless-microphone</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
         <is>
           <t>Audio - Accessories</t>
         </is>
       </c>
-      <c r="B31" s="2" t="inlineStr">
+      <c r="C31" t="inlineStr">
         <is>
           <t>AeroMic mobile wireless microphone</t>
         </is>
       </c>
-      <c r="C31" s="2" t="inlineStr">
+      <c r="D31" t="inlineStr">
         <is>
           <t>799-1499</t>
         </is>
       </c>
-      <c r="D31" s="2" t="inlineStr">
+      <c r="E31" t="inlineStr">
         <is>
           <t>/workspace/shakti-mobiles/images/interior-counter.jpg</t>
         </is>
       </c>
-      <c r="E31" s="2" t="inlineStr">
+      <c r="F31" t="inlineStr">
         <is>
           <t>Clip-on / mobile wireless mic kit for content creators</t>
         </is>
       </c>
-      <c r="F31" s="2" t="inlineStr">
+      <c r="G31" t="inlineStr">
         <is>
           <t>AeroMic box visible on lower accessory shelf.</t>
         </is>
       </c>
-      <c r="G31" s="2" t="inlineStr">
+      <c r="H31" t="inlineStr">
         <is>
           <t>Typical India retail wireless lapel mics INR 799-1499</t>
         </is>
       </c>
+      <c r="I31" t="inlineStr">
+        <is>
+          <t>2026-09-26T23:41:58+05:30</t>
+        </is>
+      </c>
+      <c r="J31" t="inlineStr">
+        <is>
+          <t>2026-09-26T23:41:58+05:30</t>
+        </is>
+      </c>
     </row>
     <row r="32">
-      <c r="A32" s="2" t="inlineStr">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>AH-031-assorted-wired-earphones</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
         <is>
           <t>Audio - Wired</t>
         </is>
       </c>
-      <c r="B32" s="2" t="inlineStr">
+      <c r="C32" t="inlineStr">
         <is>
           <t>Assorted wired earphones</t>
         </is>
       </c>
-      <c r="C32" s="2" t="inlineStr">
+      <c r="D32" t="inlineStr">
         <is>
           <t>99-499</t>
         </is>
       </c>
-      <c r="D32" s="2" t="inlineStr">
+      <c r="E32" t="inlineStr">
         <is>
           <t>/workspace/shakti-mobiles/images/cases-fashion.jpg (right shelves)</t>
         </is>
       </c>
-      <c r="E32" s="2" t="inlineStr">
+      <c r="F32" t="inlineStr">
         <is>
           <t>3.5mm / Type-C wired in-ear earphones in white retail boxes</t>
         </is>
       </c>
-      <c r="F32" s="2" t="inlineStr">
+      <c r="G32" t="inlineStr">
         <is>
           <t>White earphone diagram boxes on glass shelves next to fashion cases.</t>
         </is>
       </c>
-      <c r="G32" s="2" t="inlineStr">
+      <c r="H32" t="inlineStr">
         <is>
           <t>Typical India retail INR 99-499</t>
         </is>
       </c>
+      <c r="I32" t="inlineStr">
+        <is>
+          <t>2026-09-26T23:41:58+05:30</t>
+        </is>
+      </c>
+      <c r="J32" t="inlineStr">
+        <is>
+          <t>2026-09-26T23:41:58+05:30</t>
+        </is>
+      </c>
     </row>
     <row r="33">
-      <c r="A33" s="2" t="inlineStr">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>AH-032-fast-wall-chargers-35w-44w-65w-80w-100w</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
         <is>
           <t>Chargers</t>
         </is>
       </c>
-      <c r="B33" s="2" t="inlineStr">
+      <c r="C33" t="inlineStr">
         <is>
           <t>Fast wall chargers (35W / 44W / 65W / 80W / 100W)</t>
         </is>
       </c>
-      <c r="C33" s="2" t="inlineStr">
+      <c r="D33" t="inlineStr">
         <is>
           <t>399-1499</t>
         </is>
       </c>
-      <c r="D33" s="2" t="inlineStr">
+      <c r="E33" t="inlineStr">
         <is>
           <t>/workspace/shakti-mobiles/images/interior-counter.jpg ; cases-fashion.jpg</t>
         </is>
       </c>
-      <c r="E33" s="2" t="inlineStr">
+      <c r="F33" t="inlineStr">
         <is>
           <t>USB wall adapters labeled 35W, 44W FlashCharge, 65W SuperVOOC, 80W, 100W Super Fast on packaging</t>
         </is>
       </c>
-      <c r="F33" s="2" t="inlineStr">
+      <c r="G33" t="inlineStr">
         <is>
           <t>Wattage labels clearly visible on white charger boxes. Compatibility varies by phone brand (VOOC/PD).</t>
         </is>
       </c>
-      <c r="G33" s="2" t="inlineStr">
+      <c r="H33" t="inlineStr">
         <is>
           <t>Typical India retail GaN/fast adapters INR 399-1499 depending on wattage/brand</t>
         </is>
       </c>
+      <c r="I33" t="inlineStr">
+        <is>
+          <t>2026-09-26T23:41:58+05:30</t>
+        </is>
+      </c>
+      <c r="J33" t="inlineStr">
+        <is>
+          <t>2026-09-26T23:41:58+05:30</t>
+        </is>
+      </c>
     </row>
     <row r="34">
-      <c r="A34" s="2" t="inlineStr">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>AH-033-car-chargers-30w-pd-realme-lyne-fuel-3v</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
         <is>
           <t>Chargers</t>
         </is>
       </c>
-      <c r="B34" s="2" t="inlineStr">
+      <c r="C34" t="inlineStr">
         <is>
           <t>Car chargers (30W PD / realme / Lyne / Fuel 3V)</t>
         </is>
       </c>
-      <c r="C34" s="2" t="inlineStr">
+      <c r="D34" t="inlineStr">
         <is>
           <t>299-799</t>
         </is>
       </c>
-      <c r="D34" s="2" t="inlineStr">
+      <c r="E34" t="inlineStr">
         <is>
           <t>/workspace/shakti-mobiles/images/interior-counter.jpg</t>
         </is>
       </c>
-      <c r="E34" s="2" t="inlineStr">
+      <c r="F34" t="inlineStr">
         <is>
           <t>12V car USB chargers including 30W PD and branded realme/Lyne packs</t>
         </is>
       </c>
-      <c r="F34" s="2" t="inlineStr">
+      <c r="G34" t="inlineStr">
         <is>
           <t>Multiple car-charger boxes on mid shelves.</t>
         </is>
       </c>
-      <c r="G34" s="2" t="inlineStr">
+      <c r="H34" t="inlineStr">
         <is>
           <t>Typical India retail car chargers INR 299-799</t>
         </is>
       </c>
+      <c r="I34" t="inlineStr">
+        <is>
+          <t>2026-09-26T23:41:58+05:30</t>
+        </is>
+      </c>
+      <c r="J34" t="inlineStr">
+        <is>
+          <t>2026-09-26T23:41:58+05:30</t>
+        </is>
+      </c>
     </row>
     <row r="35">
-      <c r="A35" s="2" t="inlineStr">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>AH-034-assorted-usb-data-fast-charging-cables</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
         <is>
           <t>Cables</t>
         </is>
       </c>
-      <c r="B35" s="2" t="inlineStr">
+      <c r="C35" t="inlineStr">
         <is>
           <t>Assorted USB data / fast-charging cables</t>
         </is>
       </c>
-      <c r="C35" s="2" t="inlineStr">
+      <c r="D35" t="inlineStr">
         <is>
           <t>99-499</t>
         </is>
       </c>
-      <c r="D35" s="2" t="inlineStr">
+      <c r="E35" t="inlineStr">
         <is>
           <t>/workspace/shakti-mobiles/images/cases-fashion.jpg ; interior-counter.jpg</t>
         </is>
       </c>
-      <c r="E35" s="2" t="inlineStr">
+      <c r="F35" t="inlineStr">
         <is>
           <t>USB-A/USB-C/Lightning data and fast-charge cables in white retail boxes</t>
         </is>
       </c>
-      <c r="F35" s="2" t="inlineStr">
+      <c r="G35" t="inlineStr">
         <is>
           <t>Dense stock of cable boxes on glass shelves beside fashion cases and behind counter.</t>
         </is>
       </c>
-      <c r="G35" s="2" t="inlineStr">
+      <c r="H35" t="inlineStr">
         <is>
           <t>Typical India retail INR 99-499</t>
         </is>
       </c>
+      <c r="I35" t="inlineStr">
+        <is>
+          <t>2026-09-26T23:41:58+05:30</t>
+        </is>
+      </c>
+      <c r="J35" t="inlineStr">
+        <is>
+          <t>2026-09-26T23:41:58+05:30</t>
+        </is>
+      </c>
     </row>
     <row r="36">
-      <c r="A36" s="2" t="inlineStr">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>AH-035-realme-10000mah-power-bank</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr">
         <is>
           <t>Power Banks</t>
         </is>
       </c>
-      <c r="B36" s="2" t="inlineStr">
+      <c r="C36" t="inlineStr">
         <is>
           <t>realme 10000mAh power bank</t>
         </is>
       </c>
-      <c r="C36" s="2" t="inlineStr">
+      <c r="D36" t="inlineStr">
         <is>
           <t>599-999</t>
         </is>
       </c>
-      <c r="D36" s="2" t="inlineStr">
+      <c r="E36" t="inlineStr">
         <is>
           <t>Chat upload accessory shelves; interior-counter.jpg</t>
         </is>
       </c>
-      <c r="E36" s="2" t="inlineStr">
+      <c r="F36" t="inlineStr">
         <is>
           <t>realme yellow 10000mAh power bank (18W-33W variants common)</t>
         </is>
       </c>
-      <c r="F36" s="2" t="inlineStr">
+      <c r="G36" t="inlineStr">
         <is>
           <t>Signature yellow realme power-bank box on lower shelf.</t>
         </is>
       </c>
-      <c r="G36" s="2" t="inlineStr">
+      <c r="H36" t="inlineStr">
         <is>
           <t>https://www.flipkart.com/realme-10000-mah-power-bank-22-5-w-quick-charge-3-0/p/itm3b697fca93ba8</t>
         </is>
       </c>
+      <c r="I36" t="inlineStr">
+        <is>
+          <t>2026-09-26T23:41:58+05:30</t>
+        </is>
+      </c>
+      <c r="J36" t="inlineStr">
+        <is>
+          <t>2026-09-26T23:41:58+05:30</t>
+        </is>
+      </c>
     </row>
     <row r="37">
-      <c r="A37" s="2" t="inlineStr">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>AH-036-10000mah-power-bank-generic-multi-brand</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
         <is>
           <t>Power Banks</t>
         </is>
       </c>
-      <c r="B37" s="2" t="inlineStr">
+      <c r="C37" t="inlineStr">
         <is>
           <t>10000mAh power bank (generic / multi-brand)</t>
         </is>
       </c>
-      <c r="C37" s="2" t="inlineStr">
+      <c r="D37" t="inlineStr">
         <is>
           <t>499-999</t>
         </is>
       </c>
-      <c r="D37" s="2" t="inlineStr">
+      <c r="E37" t="inlineStr">
         <is>
           <t>/workspace/shakti-mobiles/images/interior-counter.jpg</t>
         </is>
       </c>
-      <c r="E37" s="2" t="inlineStr">
+      <c r="F37" t="inlineStr">
         <is>
           <t>10000mAh portable battery packs (black retail box also visible)</t>
         </is>
       </c>
-      <c r="F37" s="2" t="inlineStr">
+      <c r="G37" t="inlineStr">
         <is>
           <t>Additional non-realme 10000mAh box on bottom shelf.</t>
         </is>
       </c>
-      <c r="G37" s="2" t="inlineStr">
+      <c r="H37" t="inlineStr">
         <is>
           <t>Typical India retail INR 499-999</t>
         </is>
       </c>
+      <c r="I37" t="inlineStr">
+        <is>
+          <t>2026-09-26T23:41:58+05:30</t>
+        </is>
+      </c>
+      <c r="J37" t="inlineStr">
+        <is>
+          <t>2026-09-26T23:41:58+05:30</t>
+        </is>
+      </c>
     </row>
     <row r="38">
-      <c r="A38" s="2" t="inlineStr">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>AH-037-wireless-charging-pad</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr">
         <is>
           <t>Chargers</t>
         </is>
       </c>
-      <c r="B38" s="2" t="inlineStr">
+      <c r="C38" t="inlineStr">
         <is>
           <t>Wireless charging pad</t>
         </is>
       </c>
-      <c r="C38" s="2" t="inlineStr">
+      <c r="D38" t="inlineStr">
         <is>
           <t>499-999</t>
         </is>
       </c>
-      <c r="D38" s="2" t="inlineStr">
+      <c r="E38" t="inlineStr">
         <is>
           <t>/workspace/shakti-mobiles/images/interior-counter.jpg</t>
         </is>
       </c>
-      <c r="E38" s="2" t="inlineStr">
+      <c r="F38" t="inlineStr">
         <is>
           <t>Circular Qi wireless charging puck in square white retail box</t>
         </is>
       </c>
-      <c r="F38" s="2" t="inlineStr">
+      <c r="G38" t="inlineStr">
         <is>
           <t>Visible on bottom accessory shelf.</t>
         </is>
       </c>
-      <c r="G38" s="2" t="inlineStr">
+      <c r="H38" t="inlineStr">
         <is>
           <t>Typical India retail wireless pads INR 499-999</t>
         </is>
       </c>
+      <c r="I38" t="inlineStr">
+        <is>
+          <t>2026-09-26T23:41:58+05:30</t>
+        </is>
+      </c>
+      <c r="J38" t="inlineStr">
+        <is>
+          <t>2026-09-26T23:41:58+05:30</t>
+        </is>
+      </c>
     </row>
     <row r="39">
-      <c r="A39" s="2" t="inlineStr">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>AH-038-lyne-smartwatch</t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr">
         <is>
           <t>Wearables</t>
         </is>
       </c>
-      <c r="B39" s="2" t="inlineStr">
+      <c r="C39" t="inlineStr">
         <is>
           <t>LYNE smartwatch</t>
         </is>
       </c>
-      <c r="C39" s="2" t="inlineStr">
+      <c r="D39" t="inlineStr">
         <is>
           <t>999-1999</t>
         </is>
       </c>
-      <c r="D39" s="2" t="inlineStr">
+      <c r="E39" t="inlineStr">
         <is>
           <t>/workspace/shakti-mobiles/images/interior-counter.jpg</t>
         </is>
       </c>
-      <c r="E39" s="2" t="inlineStr">
+      <c r="F39" t="inlineStr">
         <is>
           <t>Square-faced smartwatch in LYNE black retail packaging; BT calling variants common in segment</t>
         </is>
       </c>
-      <c r="F39" s="2" t="inlineStr">
+      <c r="G39" t="inlineStr">
         <is>
           <t>LYNE smartwatch box clearly labeled on mid shelf. Exact model number not fully readable.</t>
         </is>
       </c>
-      <c r="G39" s="2" t="inlineStr">
+      <c r="H39" t="inlineStr">
         <is>
           <t>LYNE value smartwatch India retail typically INR 999-1999</t>
         </is>
       </c>
+      <c r="I39" t="inlineStr">
+        <is>
+          <t>2026-09-26T23:41:58+05:30</t>
+        </is>
+      </c>
+      <c r="J39" t="inlineStr">
+        <is>
+          <t>2026-09-26T23:41:58+05:30</t>
+        </is>
+      </c>
     </row>
     <row r="40">
-      <c r="A40" s="2" t="inlineStr">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>AH-039-assorted-smartwatches-multi-brand</t>
+        </is>
+      </c>
+      <c r="B40" t="inlineStr">
         <is>
           <t>Wearables</t>
         </is>
       </c>
-      <c r="B40" s="2" t="inlineStr">
+      <c r="C40" t="inlineStr">
         <is>
           <t>Assorted smartwatches (multi-brand)</t>
         </is>
       </c>
-      <c r="C40" s="2" t="inlineStr">
+      <c r="D40" t="inlineStr">
         <is>
           <t>999-2499</t>
         </is>
       </c>
-      <c r="D40" s="2" t="inlineStr">
+      <c r="E40" t="inlineStr">
         <is>
           <t>Storefront yellow banner icons; accessory shelves</t>
         </is>
       </c>
-      <c r="E40" s="2" t="inlineStr">
+      <c r="F40" t="inlineStr">
         <is>
           <t>Smartwatches advertised on store banner (icons) and stocked in square boxes</t>
         </is>
       </c>
-      <c r="F40" s="2" t="inlineStr">
+      <c r="G40" t="inlineStr">
         <is>
           <t>Banner promotes smartwatches; multiple square watch boxes on shelves beyond LYNE.</t>
         </is>
       </c>
-      <c r="G40" s="2" t="inlineStr">
+      <c r="H40" t="inlineStr">
         <is>
           <t>Typical India retail entry smartwatches INR 999-2499</t>
+        </is>
+      </c>
+      <c r="I40" t="inlineStr">
+        <is>
+          <t>2026-09-26T23:41:58+05:30</t>
+        </is>
+      </c>
+      <c r="J40" t="inlineStr">
+        <is>
+          <t>2026-09-26T23:41:58+05:30</t>
         </is>
       </c>
     </row>
@@ -1957,6 +2561,951 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:E40"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="28" customWidth="1" min="1" max="1"/>
+    <col width="12" customWidth="1" min="2" max="2"/>
+    <col width="20" customWidth="1" min="3" max="3"/>
+    <col width="60" customWidth="1" min="4" max="4"/>
+    <col width="28" customWidth="1" min="5" max="5"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="5" t="inlineStr">
+        <is>
+          <t>product_id</t>
+        </is>
+      </c>
+      <c r="B1" s="5" t="inlineStr">
+        <is>
+          <t>change_type</t>
+        </is>
+      </c>
+      <c r="C1" s="5" t="inlineStr">
+        <is>
+          <t>old_value</t>
+        </is>
+      </c>
+      <c r="D1" s="5" t="inlineStr">
+        <is>
+          <t>new_value</t>
+        </is>
+      </c>
+      <c r="E1" s="5" t="inlineStr">
+        <is>
+          <t>timestamp</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>AH-001-infinix-smart-8-hd-shiny-gold-3gb-64gb</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>added</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr"/>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>{"Category": "Smartphones", "Product Name": "Infinix SMART 8 HD (Shiny Gold, 3GB/64GB)", "Price (INR)": "6699", "Image Source/URL": "/workspace/shakti-mobiles/images/products/phone-4g.jpg", "Specs": "6.6\" HD+ IPS; Unisoc T606; 3GB RAM / 64GB ROM (expandable to 2TB); 13MP + AI rear, 8MP front; 5000mAh; 10W; Dual SIM 4G", "Notes": "Verified Flipkart listing. Color Shiny Gold visible in store product photo. Alternate images: phone-4g-infinix.jpg, phone-4g-alt.jpg.", "Source Links": "https://www.flipkart.com/infinix-smart-8-hd-shiny-gold-64-gb/p/itm709d885ba6ac1?pid=MOBGVAPXG4WHFR9M ; https://infinixmobiles.in/products/smart-8-hd", "id": "AH-001-infinix-smart-8-hd-shiny-gold-3gb-64gb"}</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>2026-09-26T23:41:58+05:30</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>AH-002-poco-c75-5g-aqua-bliss-4gb-64gb</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>added</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr"/>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>{"Category": "Smartphones", "Product Name": "POCO C75 5G (Aqua Bliss, 4GB/64GB)", "Price (INR)": "10999", "Image Source/URL": "/workspace/shakti-mobiles/images/products/phone-5g-try1.jpg", "Specs": "6.88\" HD+ 120Hz; Snapdragon 4s Gen 2 5G; 4GB/64GB (expandable 1TB); 50MP Sony rear, 5MP front; 5160mAh; Dual SIM", "Notes": "Prefer phone-5g-try1.jpg over phone-5g.jpg per catalog guidance. Flipkart ~INR 10,999 (bank offer may lower).", "Source Links": "https://www.flipkart.com/poco-c75-5g-aqua-bliss-64-gb/p/itm10b3f6f1bc616", "id": "AH-002-poco-c75-5g-aqua-bliss-4gb-64gb"}</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>2026-09-26T23:41:58+05:30</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>AH-003-lava-bold-n4-lite-empire-gold-3gb-32gb</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>added</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr"/>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>{"Category": "Smartphones", "Product Name": "Lava Bold N4 Lite (Empire Gold, 3GB/32GB)", "Price (INR)": "8399", "Image Source/URL": "/workspace/shakti-mobiles/images/products/phone-samsung-f05.jpg", "Specs": "6.56\" qHD; Unisoc 9863A; 3GB+3GB virtual RAM / 32GB ROM (expandable 64GB); 8MP rear, 5MP front; 5000mAh; 10W; Android 16 Go; MIL-STD-810H", "Notes": "File named phone-samsung-f05.jpg but image content is Lava Bold N4 Lite (LAVA logo + BOLD N4 LITE on screen). Same asset as phone-4g-samsung-amz.jpg. Amazon.in exclusive; ~INR 7,999–8,399.", "Source Links": "https://www.amazon.in/Lava-Storage-Display-Fingerprint-Phone-Cover/dp/B0HDPDGKJ4 ; https://www.91mobiles.com/lava-bold-n4-lite-4g-price-in-india", "id": "AH-003-lava-bold-n4-lite-empire-gold-3gb-32gb"}</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>2026-09-26T23:41:58+05:30</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>AH-004-samsung-galaxy-f05-4gb-64gb</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>added</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr"/>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>{"Category": "Smartphones", "Product Name": "Samsung Galaxy F05 (4GB/64GB)", "Price (INR)": "6499", "Image Source/URL": "Store brand signage (Samsung listed); no dedicated clear F05 product photo in inspected set", "Specs": "6.74\" HD+; Helio G85; 4GB/64GB (expandable 1TB); 50MP+2MP rear, 8MP front; 5000mAh; 25W; Android 14; Dual SIM 4G", "Notes": "Store sells Samsung (signage). Prior catalog guidance confirmed ~INR 6,499 Flipkart/Smartprix. Dedicated image file was mislabeled (see Lava Bold N4 Lite row).", "Source Links": "https://www.flipkart.com/samsung-galaxy-f05-twilight-blue-64-gb/p/itm84a914081ab93 ; https://www.smartprix.com/mobiles/samsung-galaxy-f05-ppd1u4z3r099", "id": "AH-004-samsung-galaxy-f05-4gb-64gb"}</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>2026-09-26T23:41:58+05:30</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>AH-005-redmi-a3-assorted-variants</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>added</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr"/>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>{"Category": "Smartphones", "Product Name": "REDMI A3 (assorted variants)", "Price (INR)": "6998-7340", "Image Source/URL": "/workspace/shakti-mobiles/images/service-counter.jpg ; chat upload interior counter", "Specs": "Budget Redmi A-series; typical configs 3GB/64GB to 6GB/128GB; Dual SIM 4G", "Notes": "Red retail box clearly visible on glass counter labeled REDMI A3. Exact RAM/storage of in-store unit not readable; price range from Flipkart variants.", "Source Links": "https://pricehistory.app/p/redmi-a3-lake-blue-64-gb-3-TTlxopmb ; https://www.flipkart.com/redmi-a3-lake-blue-128-gb/p/itmbe3bd4f2bebed", "id": "AH-005-redmi-a3-assorted-variants"}</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>2026-09-26T23:41:58+05:30</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>AH-006-realme-smartphone-boxed-model-unclear</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>added</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr"/>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>{"Category": "Smartphones", "Product Name": "realme smartphone (boxed — model unclear)", "Price (INR)": "Varies", "Image Source/URL": "/workspace/shakti-mobiles/images/service-counter.jpg", "Specs": "realme branded yellow retail box on counter; exact model text not fully legible (possible C-series)", "Notes": "Could not confidently identify exact model from box photo. Store carries realme (signage + accessories).", "Source Links": "https://www.realme.com/in/", "id": "AH-006-realme-smartphone-boxed-model-unclear"}</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>2026-09-26T23:41:58+05:30</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>AH-007-nokia-feature-phone-105-110-class</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>added</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr"/>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>{"Category": "Feature Phones", "Product Name": "Nokia feature phone (105/110-class)", "Price (INR)": "999-1589", "Image Source/URL": "Chat upload service/accessory shelves (Nokia blue box)", "Specs": "Keypad feature phone; Dual SIM options typical for Nokia 105 Classic / related", "Notes": "Small blue Nokia retail box visible on lower accessory shelf. Exact SKU (105 vs 110) not readable at distance.", "Source Links": "https://pricehunt.com/mobiles/nokia-105.php", "id": "AH-007-nokia-feature-phone-105-110-class"}</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>2026-09-26T23:41:58+05:30</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>AH-008-assorted-fashion-back-covers-cartoon-glitter-but</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>added</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr"/>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>{"Category": "Phone Cases", "Product Name": "Assorted fashion back covers (cartoon / glitter / butterfly)", "Price (INR)": "99-499", "Image Source/URL": "/workspace/shakti-mobiles/images/cases-fashion.jpg ; chat fashion-case wall", "Specs": "TPU/silicone fashion cases; themes include Hello Kitty, Tom &amp; Jerry, Labubu, butterflies, glitter/quicksand, rhinestones", "Notes": "In-store assortment; price varies by model and style. Packaged as Fashion Case.", "Source Links": "Typical India retail for generic fashion covers INR 99-499", "id": "AH-008-assorted-fashion-back-covers-cartoon-glitter-but"}</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>2026-09-26T23:41:58+05:30</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>AH-009-geometric-diamond-facet-fashion-cases</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>added</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr"/>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>{"Category": "Phone Cases", "Product Name": "Geometric / diamond-facet fashion cases", "Price (INR)": "149-499", "Image Source/URL": "/workspace/shakti-mobiles/images/cases-fashion.jpg ; /workspace/shakti-mobiles/images/cases-wall.jpg", "Specs": "3D crystalline / mosaic facet hard-back fashion covers in pink, purple, gold, black", "Notes": "In-store assortment; price varies.", "Source Links": "Typical India retail INR 149-499", "id": "AH-009-geometric-diamond-facet-fashion-cases"}</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>2026-09-26T23:41:58+05:30</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>AH-010-transparent-tpu-clear-covers</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>added</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr"/>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>{"Category": "Phone Cases", "Product Name": "Transparent TPU / clear covers", "Price (INR)": "99-299", "Image Source/URL": "/workspace/shakti-mobiles/images/cases-wall.jpg ; interior counter glass case", "Specs": "Clear TPU/PC protective backs; some with glitter insert", "Notes": "Large wall inventory of basic clear covers. In-store assortment; price varies.", "Source Links": "Typical India retail INR 99-299", "id": "AH-010-transparent-tpu-clear-covers"}</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>2026-09-26T23:41:58+05:30</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>AH-011-lustre-rugged-matte-tpu-cases</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>added</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr"/>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>{"Category": "Phone Cases", "Product Name": "Lustre rugged / matte TPU cases", "Price (INR)": "199-499", "Image Source/URL": "/workspace/shakti-mobiles/images/cases-wall.jpg", "Specs": "Lustre-branded yellow/black hang packs; solid black/navy/red matte or textured protective covers", "Notes": "Brand Lustre visible on packaging. Premium end of in-store case range.", "Source Links": "Typical India retail for branded rugged TPU INR 199-499", "id": "AH-011-lustre-rugged-matte-tpu-cases"}</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>2026-09-26T23:41:58+05:30</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>AH-012-magsafe-compatible-clear-cases</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>added</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr"/>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>{"Category": "Phone Cases", "Product Name": "MagSafe-compatible clear cases", "Price (INR)": "299-499", "Image Source/URL": "/workspace/shakti-mobiles/images/cases-wall.jpg", "Specs": "Clear cases with white circular MagSafe-style magnetic ring", "Notes": "Multiple MagSafe ring cases on wall pegs. In-store assortment.", "Source Links": "Typical India retail INR 299-499", "id": "AH-012-magsafe-compatible-clear-cases"}</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>2026-09-26T23:41:58+05:30</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>AH-013-puffer-quilted-jacket-style-cases</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>added</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr"/>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>{"Category": "Phone Cases", "Product Name": "Puffer / quilted jacket-style cases", "Price (INR)": "249-499", "Image Source/URL": "/workspace/shakti-mobiles/images/cases-wall.jpg", "Specs": "Quilted puffer textured soft cases, typically black", "Notes": "At least two puffer-style units visible on cases wall.", "Source Links": "Typical India retail INR 249-499", "id": "AH-013-puffer-quilted-jacket-style-cases"}</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>2026-09-26T23:41:58+05:30</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>AH-014-designer-character-graphic-cases-disney-luxury-m</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>added</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr"/>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>{"Category": "Phone Cases", "Product Name": "Designer / character graphic cases (Disney, luxury-motif prints)", "Price (INR)": "149-499", "Image Source/URL": "/workspace/shakti-mobiles/images/cases-wall.jpg", "Specs": "Printed graphic covers including Disney (Donald Duck, Minnie), Chanel/Dior-style motifs, Starbucks-style, Ferrari-style logos", "Notes": "In-store assortment of printed designer-look cases; unofficial motif prints common in local retail.", "Source Links": "Typical India retail INR 149-499", "id": "AH-014-designer-character-graphic-cases-disney-luxury-m"}</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>2026-09-26T23:41:58+05:30</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>AH-015-yellow-waterproof-phone-pouches-dry-bags-with-la</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>added</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr"/>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>{"Category": "Phone Accessories", "Product Name": "Yellow waterproof phone pouches (dry bags with lanyard)", "Price (INR)": "99-249", "Image Source/URL": "/workspace/shakti-mobiles/images/cases-wall.jpg", "Specs": "Transparent yellow waterproof dry bag with matching neck lanyard; universal phone size", "Notes": "Cluster hanging on far-right of cases wall. In-store assortment.", "Source Links": "Typical India retail waterproof pouches INR 99-249", "id": "AH-015-yellow-waterproof-phone-pouches-dry-bags-with-la"}</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>2026-09-26T23:41:58+05:30</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>AH-016-tempered-glass-screen-protector</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>added</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr"/>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>{"Category": "Screen Protection", "Product Name": "Tempered glass screen protector", "Price (INR)": "100", "Image Source/URL": "/workspace/shakti-mobiles/images/storefront-1.jpg ; storefront-2.jpg", "Specs": "Generic tempered glass; store advertises base price INR 100", "Notes": "Window card: ANGAALA HUB TEMPER GLASS INR 100. Model-specific pricing may vary.", "Source Links": "In-store advertised price INR 100", "id": "AH-016-tempered-glass-screen-protector"}</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>2026-09-26T23:41:58+05:30</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>AH-017-custom-cut-screen-guard-uv-film-auto-laminate-ma</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>added</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr"/>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>{"Category": "Screen Protection", "Product Name": "Custom-cut screen guard / UV film (auto laminate machine)", "Price (INR)": "149-499", "Image Source/URL": "Chat upload counter (REPROTECT UV vacuum film applicator); storefront yellow banner", "Specs": "Sticker/screen guard cutting machine with auto laminate; UV curing lamp; matte/glossy options; mobile + laptop skins", "Notes": "REPROTECT Mobile UV vacuum film applicator under glass counter. Service + product hybrid.", "Source Links": "Typical India custom hydrogel/UV film installs INR 149-499", "id": "AH-017-custom-cut-screen-guard-uv-film-auto-laminate-ma"}</t>
+        </is>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>2026-09-26T23:41:58+05:30</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>AH-018-laptop-and-mobile-skins</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>added</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr"/>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>{"Category": "Screen Protection", "Product Name": "Laptop and mobile skins", "Price (INR)": "149-499", "Image Source/URL": "/workspace/shakti-mobiles/images/storefront-1.jpg", "Specs": "Adhesive decorative/protective skins for phones and laptops", "Notes": "Blue flyer in window: Laptop and Mobile Skins.", "Source Links": "Typical India retail skins INR 149-499", "id": "AH-018-laptop-and-mobile-skins"}</t>
+        </is>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>2026-09-26T23:41:58+05:30</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>AH-019-boat-rockerz-450-on-ear-bluetooth</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>added</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr"/>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>{"Category": "Audio - Headphones", "Product Name": "boAt Rockerz 450 (on-ear Bluetooth)", "Price (INR)": "1699-1899", "Image Source/URL": "/workspace/shakti-mobiles/images/interior-counter.jpg", "Specs": "40mm drivers; up to ~15H playback; Bluetooth + AUX; on-ear", "Notes": "White boAt over-ear/on-ear box visible on top accessory shelf.", "Source Links": "https://www.boat-lifestyle.com/products/rockerz-450 ; https://www.flipkart.com/boat-rockerz-450-40mm-drivers-15h-battery-stream-ad-free-music-via-app-bluetooth/p/itm077a566bd128b", "id": "AH-019-boat-rockerz-450-on-ear-bluetooth"}</t>
+        </is>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>2026-09-26T23:41:58+05:30</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>AH-020-boat-shine-assorted-over-ear-headphones</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>added</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr"/>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>{"Category": "Audio - Headphones", "Product Name": "boAt Shine / assorted over-ear headphones", "Price (INR)": "1499-2499", "Image Source/URL": "Chat upload accessory shelves; interior-counter.jpg", "Specs": "Over-ear wireless headphones; boAt Shine white/silver packaging among others (P9/P3 wireless headsets also stocked)", "Notes": "Multiple over-ear boxes on top shelf including boAt Shine, P9 Wireless Headset, Noise headphones.", "Source Links": "Typical India retail over-ear Bluetooth INR 1499-2499", "id": "AH-020-boat-shine-assorted-over-ear-headphones"}</t>
+        </is>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>2026-09-26T23:41:58+05:30</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>AH-021-boat-rockerz-series-wireless-neckbands-assorted</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>added</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr"/>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>{"Category": "Audio - Neckbands", "Product Name": "boAt Rockerz series wireless neckbands (assorted)", "Price (INR)": "799-1499", "Image Source/URL": "/workspace/shakti-mobiles/images/interior-counter.jpg ; service-counter.jpg", "Specs": "Wireless neckband earphones; Rockerz / Rockerz Turbo Power lineup; Bluetooth", "Notes": "Many slim boAt Rockerz boxes; Hardik Pandya Rockerz Turbo Power standee visible. Also Captain / Vibration branded neckband boxes.", "Source Links": "https://www.boat-lifestyle.com/ ; Flipkart boAt Rockerz listings typically INR 799-1499", "id": "AH-021-boat-rockerz-series-wireless-neckbands-assorted"}</t>
+        </is>
+      </c>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>2026-09-26T23:41:58+05:30</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>AH-022-noise-wireless-neckband</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>added</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr"/>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>{"Category": "Audio - Neckbands", "Product Name": "Noise wireless neckband", "Price (INR)": "999-1499", "Image Source/URL": "Chat upload accessory shelves; interior-counter.jpg", "Specs": "Noise-branded wireless neckband earphones", "Notes": "Light blue / black Noise box on audio shelf. Exact model name not fully readable.", "Source Links": "https://www.smartprix.com/mobile_headphones/noise-nerve-wireless-neckband-ppd146xzqfsb", "id": "AH-022-noise-wireless-neckband"}</t>
+        </is>
+      </c>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>2026-09-26T23:41:58+05:30</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>AH-023-ditto-rockers-13-pro-neckbands</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>added</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr"/>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>{"Category": "Audio - Neckbands", "Product Name": "DITTO / Rockers 13 Pro neckbands", "Price (INR)": "499-999", "Image Source/URL": "/workspace/shakti-mobiles/images/interior-counter.jpg", "Specs": "Value wireless neckbands; Rockers 13 Pro box advertises long playback (e.g. 450h claim on pack)", "Notes": "Local/value brands alongside boAt on same shelves.", "Source Links": "Typical India retail value neckbands INR 499-999", "id": "AH-023-ditto-rockers-13-pro-neckbands"}</t>
+        </is>
+      </c>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>2026-09-26T23:41:58+05:30</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>AH-024-realme-buds-wireless-buds-classic-neckband-and-w</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>added</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr"/>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>{"Category": "Audio - Neckbands", "Product Name": "realme Buds Wireless / Buds Classic (neckband and wired)", "Price (INR)": "699-1499", "Image Source/URL": "/workspace/shakti-mobiles/images/interior-counter.jpg", "Specs": "realme yellow retail audio boxes; Buds Classic wired and Buds Wireless neckband variants stocked", "Notes": "Multiple signature yellow realme audio boxes on charger/TWS shelf row.", "Source Links": "Flipkart realme Buds listings typically INR 699-1499", "id": "AH-024-realme-buds-wireless-buds-classic-neckband-and-w"}</t>
+        </is>
+      </c>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>2026-09-26T23:41:58+05:30</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>AH-025-oneplus-nord-buds-2r-buds-2r</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>added</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr"/>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>{"Category": "Audio - TWS Earbuds", "Product Name": "OnePlus Nord Buds 2r (Buds 2r)", "Price (INR)": "1649-2199", "Image Source/URL": "Chat upload accessory shelves; interior-counter.jpg", "Specs": "True wireless earbuds; OnePlus Buds 2r / Nord Buds 2R packaging", "Notes": "White/blue Buds 2r box visible among TWS row.", "Source Links": "https://www.smartprix.com/mobile_headphones/oneplus-nord-buds-2r-true-wireless-earbuds-ppd15t83jbh5", "id": "AH-025-oneplus-nord-buds-2r-buds-2r"}</t>
+        </is>
+      </c>
+      <c r="E26" t="inlineStr">
+        <is>
+          <t>2026-09-26T23:41:58+05:30</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>AH-026-boat-airdopes-tws-assorted-models</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>added</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr"/>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>{"Category": "Audio - TWS Earbuds", "Product Name": "boAt Airdopes TWS (assorted models)", "Price (INR)": "799-1999", "Image Source/URL": "/workspace/shakti-mobiles/images/interior-counter.jpg", "Specs": "boAt Airdopes true wireless earbuds; multiple SKUs on shelf", "Notes": "Several small Airdopes boxes on TWS shelf. Exact model mix varies.", "Source Links": "https://www.boat-lifestyle.com/ ; Flipkart Airdopes typically INR 799-1999", "id": "AH-026-boat-airdopes-tws-assorted-models"}</t>
+        </is>
+      </c>
+      <c r="E27" t="inlineStr">
+        <is>
+          <t>2026-09-26T23:41:58+05:30</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>AH-027-u-i-m10-generic-tws-earbuds</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>added</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr"/>
+      <c r="D28" t="inlineStr">
+        <is>
+          <t>{"Category": "Audio - TWS Earbuds", "Product Name": "U&amp;i / M10 / generic TWS earbuds", "Price (INR)": "499-999", "Image Source/URL": "/workspace/shakti-mobiles/images/interior-counter.jpg", "Specs": "Value TWS earbuds (U&amp;i branded and M10-style packs)", "Notes": "Value TWS next to branded boAt/OnePlus stock.", "Source Links": "Typical India retail generic TWS INR 499-999", "id": "AH-027-u-i-m10-generic-tws-earbuds"}</t>
+        </is>
+      </c>
+      <c r="E28" t="inlineStr">
+        <is>
+          <t>2026-09-26T23:41:58+05:30</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>AH-028-lyne-jukebox-18-blaster-party-speaker</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>added</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr"/>
+      <c r="D29" t="inlineStr">
+        <is>
+          <t>{"Category": "Audio - Speakers", "Product Name": "LYNE JukeBox 18 / Blaster party speaker", "Price (INR)": "1899-1999", "Image Source/URL": "/workspace/shakti-mobiles/images/storefront-1.jpg ; storefront-2.jpg", "Specs": "~30-50W wireless party speaker; dual drivers; RGB lighting; Bluetooth; some kits include mic", "Notes": "Large LYNE JukeBox / Blaster boxes in front window. JukeBox 18 Pro launch around INR 1999.", "Source Links": "https://lyneoriginals.com/products/jukebox-18 ; https://www.fonearena.com/blog/488457/lyne-blaster-series-jukebox-18-pro-price-features.html", "id": "AH-028-lyne-jukebox-18-blaster-party-speaker"}</t>
+        </is>
+      </c>
+      <c r="E29" t="inlineStr">
+        <is>
+          <t>2026-09-26T23:41:58+05:30</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>AH-029-lyne-blast-max-large-portable-bluetooth-speaker</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>added</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr"/>
+      <c r="D30" t="inlineStr">
+        <is>
+          <t>{"Category": "Audio - Speakers", "Product Name": "LYNE BLAST MAX / large portable Bluetooth speaker", "Price (INR)": "1499-2499", "Image Source/URL": "/workspace/shakti-mobiles/images/storefront-1.jpg", "Specs": "Large vertical portable Bluetooth speaker; dual-woofer party style with RGB rings (window display)", "Notes": "BLAST MAX and similar large speaker boxes in storefront window.", "Source Links": "LYNE / local portable speaker retail typically INR 1499-2499", "id": "AH-029-lyne-blast-max-large-portable-bluetooth-speaker"}</t>
+        </is>
+      </c>
+      <c r="E30" t="inlineStr">
+        <is>
+          <t>2026-09-26T23:41:58+05:30</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>AH-030-aeromic-mobile-wireless-microphone</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>added</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr"/>
+      <c r="D31" t="inlineStr">
+        <is>
+          <t>{"Category": "Audio - Accessories", "Product Name": "AeroMic mobile wireless microphone", "Price (INR)": "799-1499", "Image Source/URL": "/workspace/shakti-mobiles/images/interior-counter.jpg", "Specs": "Clip-on / mobile wireless mic kit for content creators", "Notes": "AeroMic box visible on lower accessory shelf.", "Source Links": "Typical India retail wireless lapel mics INR 799-1499", "id": "AH-030-aeromic-mobile-wireless-microphone"}</t>
+        </is>
+      </c>
+      <c r="E31" t="inlineStr">
+        <is>
+          <t>2026-09-26T23:41:58+05:30</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>AH-031-assorted-wired-earphones</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>added</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr"/>
+      <c r="D32" t="inlineStr">
+        <is>
+          <t>{"Category": "Audio - Wired", "Product Name": "Assorted wired earphones", "Price (INR)": "99-499", "Image Source/URL": "/workspace/shakti-mobiles/images/cases-fashion.jpg (right shelves)", "Specs": "3.5mm / Type-C wired in-ear earphones in white retail boxes", "Notes": "White earphone diagram boxes on glass shelves next to fashion cases.", "Source Links": "Typical India retail INR 99-499", "id": "AH-031-assorted-wired-earphones"}</t>
+        </is>
+      </c>
+      <c r="E32" t="inlineStr">
+        <is>
+          <t>2026-09-26T23:41:58+05:30</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>AH-032-fast-wall-chargers-35w-44w-65w-80w-100w</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>added</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr"/>
+      <c r="D33" t="inlineStr">
+        <is>
+          <t>{"Category": "Chargers", "Product Name": "Fast wall chargers (35W / 44W / 65W / 80W / 100W)", "Price (INR)": "399-1499", "Image Source/URL": "/workspace/shakti-mobiles/images/interior-counter.jpg ; cases-fashion.jpg", "Specs": "USB wall adapters labeled 35W, 44W FlashCharge, 65W SuperVOOC, 80W, 100W Super Fast on packaging", "Notes": "Wattage labels clearly visible on white charger boxes. Compatibility varies by phone brand (VOOC/PD).", "Source Links": "Typical India retail GaN/fast adapters INR 399-1499 depending on wattage/brand", "id": "AH-032-fast-wall-chargers-35w-44w-65w-80w-100w"}</t>
+        </is>
+      </c>
+      <c r="E33" t="inlineStr">
+        <is>
+          <t>2026-09-26T23:41:58+05:30</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>AH-033-car-chargers-30w-pd-realme-lyne-fuel-3v</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>added</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr"/>
+      <c r="D34" t="inlineStr">
+        <is>
+          <t>{"Category": "Chargers", "Product Name": "Car chargers (30W PD / realme / Lyne / Fuel 3V)", "Price (INR)": "299-799", "Image Source/URL": "/workspace/shakti-mobiles/images/interior-counter.jpg", "Specs": "12V car USB chargers including 30W PD and branded realme/Lyne packs", "Notes": "Multiple car-charger boxes on mid shelves.", "Source Links": "Typical India retail car chargers INR 299-799", "id": "AH-033-car-chargers-30w-pd-realme-lyne-fuel-3v"}</t>
+        </is>
+      </c>
+      <c r="E34" t="inlineStr">
+        <is>
+          <t>2026-09-26T23:41:58+05:30</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>AH-034-assorted-usb-data-fast-charging-cables</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>added</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr"/>
+      <c r="D35" t="inlineStr">
+        <is>
+          <t>{"Category": "Cables", "Product Name": "Assorted USB data / fast-charging cables", "Price (INR)": "99-499", "Image Source/URL": "/workspace/shakti-mobiles/images/cases-fashion.jpg ; interior-counter.jpg", "Specs": "USB-A/USB-C/Lightning data and fast-charge cables in white retail boxes", "Notes": "Dense stock of cable boxes on glass shelves beside fashion cases and behind counter.", "Source Links": "Typical India retail INR 99-499", "id": "AH-034-assorted-usb-data-fast-charging-cables"}</t>
+        </is>
+      </c>
+      <c r="E35" t="inlineStr">
+        <is>
+          <t>2026-09-26T23:41:58+05:30</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>AH-035-realme-10000mah-power-bank</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>added</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr"/>
+      <c r="D36" t="inlineStr">
+        <is>
+          <t>{"Category": "Power Banks", "Product Name": "realme 10000mAh power bank", "Price (INR)": "599-999", "Image Source/URL": "Chat upload accessory shelves; interior-counter.jpg", "Specs": "realme yellow 10000mAh power bank (18W-33W variants common)", "Notes": "Signature yellow realme power-bank box on lower shelf.", "Source Links": "https://www.flipkart.com/realme-10000-mah-power-bank-22-5-w-quick-charge-3-0/p/itm3b697fca93ba8", "id": "AH-035-realme-10000mah-power-bank"}</t>
+        </is>
+      </c>
+      <c r="E36" t="inlineStr">
+        <is>
+          <t>2026-09-26T23:41:58+05:30</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>AH-036-10000mah-power-bank-generic-multi-brand</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>added</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr"/>
+      <c r="D37" t="inlineStr">
+        <is>
+          <t>{"Category": "Power Banks", "Product Name": "10000mAh power bank (generic / multi-brand)", "Price (INR)": "499-999", "Image Source/URL": "/workspace/shakti-mobiles/images/interior-counter.jpg", "Specs": "10000mAh portable battery packs (black retail box also visible)", "Notes": "Additional non-realme 10000mAh box on bottom shelf.", "Source Links": "Typical India retail INR 499-999", "id": "AH-036-10000mah-power-bank-generic-multi-brand"}</t>
+        </is>
+      </c>
+      <c r="E37" t="inlineStr">
+        <is>
+          <t>2026-09-26T23:41:58+05:30</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>AH-037-wireless-charging-pad</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>added</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr"/>
+      <c r="D38" t="inlineStr">
+        <is>
+          <t>{"Category": "Chargers", "Product Name": "Wireless charging pad", "Price (INR)": "499-999", "Image Source/URL": "/workspace/shakti-mobiles/images/interior-counter.jpg", "Specs": "Circular Qi wireless charging puck in square white retail box", "Notes": "Visible on bottom accessory shelf.", "Source Links": "Typical India retail wireless pads INR 499-999", "id": "AH-037-wireless-charging-pad"}</t>
+        </is>
+      </c>
+      <c r="E38" t="inlineStr">
+        <is>
+          <t>2026-09-26T23:41:58+05:30</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>AH-038-lyne-smartwatch</t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>added</t>
+        </is>
+      </c>
+      <c r="C39" t="inlineStr"/>
+      <c r="D39" t="inlineStr">
+        <is>
+          <t>{"Category": "Wearables", "Product Name": "LYNE smartwatch", "Price (INR)": "999-1999", "Image Source/URL": "/workspace/shakti-mobiles/images/interior-counter.jpg", "Specs": "Square-faced smartwatch in LYNE black retail packaging; BT calling variants common in segment", "Notes": "LYNE smartwatch box clearly labeled on mid shelf. Exact model number not fully readable.", "Source Links": "LYNE value smartwatch India retail typically INR 999-1999", "id": "AH-038-lyne-smartwatch"}</t>
+        </is>
+      </c>
+      <c r="E39" t="inlineStr">
+        <is>
+          <t>2026-09-26T23:41:58+05:30</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>AH-039-assorted-smartwatches-multi-brand</t>
+        </is>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>added</t>
+        </is>
+      </c>
+      <c r="C40" t="inlineStr"/>
+      <c r="D40" t="inlineStr">
+        <is>
+          <t>{"Category": "Wearables", "Product Name": "Assorted smartwatches (multi-brand)", "Price (INR)": "999-2499", "Image Source/URL": "Storefront yellow banner icons; accessory shelves", "Specs": "Smartwatches advertised on store banner (icons) and stocked in square boxes", "Notes": "Banner promotes smartwatches; multiple square watch boxes on shelves beyond LYNE.", "Source Links": "Typical India retail entry smartwatches INR 999-2499", "id": "AH-039-assorted-smartwatches-multi-brand"}</t>
+        </is>
+      </c>
+      <c r="E40" t="inlineStr">
+        <is>
+          <t>2026-09-26T23:41:58+05:30</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -2201,7 +3750,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>

</xml_diff>